<commit_message>
Add Capital Invested and Market Value columns to 80-delta sheet
Inserts two new columns (J, K) after Total Cost showing cumulative
portfolio cost basis and BS-modeled market value at each trade's entry
date. Uses historical prices from yfinance for past rows and live
prices for today's rows.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Strategies/80-Delta Call Strategy/position_tracker.xlsx
+++ b/Strategies/80-Delta Call Strategy/position_tracker.xlsx
@@ -639,7 +639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y40"/>
+  <dimension ref="A1:AA40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -651,22 +651,24 @@
     <col width="5" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="9" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="13" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="10" customWidth="1" min="22" max="22"/>
-    <col width="13" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -679,7 +681,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last Updated: 2026-03-03 13:57:12  |  SPY: $681.09  |  QQQ: $602.48</t>
+          <t>Last Updated: 2026-03-03 14:12:14  |  SPY: $679.98  |  QQQ: $601.36</t>
         </is>
       </c>
     </row>
@@ -877,80 +879,90 @@
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
+          <t>Capital Invested</t>
+        </is>
+      </c>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>Market Value</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
           <t>Delta@Entry</t>
         </is>
       </c>
-      <c r="K19" s="6" t="inlineStr">
+      <c r="M19" s="6" t="inlineStr">
         <is>
           <t>DTE@Entry</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="N19" s="6" t="inlineStr">
         <is>
           <t>SPY@Entry</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
+      <c r="O19" s="6" t="inlineStr">
         <is>
           <t>SMA200@Entry</t>
         </is>
       </c>
-      <c r="N19" s="6" t="inlineStr">
+      <c r="P19" s="6" t="inlineStr">
         <is>
           <t>Current Price</t>
         </is>
       </c>
-      <c r="O19" s="6" t="inlineStr">
+      <c r="Q19" s="6" t="inlineStr">
         <is>
           <t>Current Value</t>
         </is>
       </c>
-      <c r="P19" s="6" t="inlineStr">
+      <c r="R19" s="6" t="inlineStr">
         <is>
           <t>Cur Delta</t>
         </is>
       </c>
-      <c r="Q19" s="6" t="inlineStr">
+      <c r="S19" s="6" t="inlineStr">
         <is>
           <t>Cur DTE</t>
         </is>
       </c>
-      <c r="R19" s="6" t="inlineStr">
+      <c r="T19" s="6" t="inlineStr">
         <is>
           <t>Unreal P&amp;L ($)</t>
         </is>
       </c>
-      <c r="S19" s="6" t="inlineStr">
+      <c r="U19" s="6" t="inlineStr">
         <is>
           <t>Unreal P&amp;L (%)</t>
         </is>
       </c>
-      <c r="T19" s="6" t="inlineStr">
+      <c r="V19" s="6" t="inlineStr">
         <is>
           <t>Target Price</t>
         </is>
       </c>
-      <c r="U19" s="6" t="inlineStr">
+      <c r="W19" s="6" t="inlineStr">
         <is>
           <t>% To Target</t>
         </is>
       </c>
-      <c r="V19" s="6" t="inlineStr">
+      <c r="X19" s="6" t="inlineStr">
         <is>
           <t>Days Held</t>
         </is>
       </c>
-      <c r="W19" s="6" t="inlineStr">
+      <c r="Y19" s="6" t="inlineStr">
         <is>
           <t>Max Hold Date</t>
         </is>
       </c>
-      <c r="X19" s="6" t="inlineStr">
+      <c r="Z19" s="6" t="inlineStr">
         <is>
           <t>Days Remaining</t>
         </is>
       </c>
-      <c r="Y19" s="6" t="inlineStr">
+      <c r="AA19" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -992,54 +1004,60 @@
       <c r="I20" s="9" t="n">
         <v>51600</v>
       </c>
-      <c r="J20" s="11" t="n">
+      <c r="J20" s="9" t="n">
+        <v>51600</v>
+      </c>
+      <c r="K20" s="9" t="n">
+        <v>53761.53242392735</v>
+      </c>
+      <c r="L20" s="11" t="n">
         <v>0.74</v>
       </c>
-      <c r="K20" s="7" t="n">
+      <c r="M20" s="7" t="n">
         <v>135</v>
       </c>
-      <c r="L20" s="9" t="n">
+      <c r="N20" s="9" t="n">
         <v>687</v>
       </c>
-      <c r="M20" s="9" t="n">
+      <c r="O20" s="9" t="n">
         <v>640</v>
       </c>
-      <c r="N20" s="10" t="n">
-        <v>43.42996547173817</v>
-      </c>
-      <c r="O20" s="9" t="n">
-        <v>43429.96547173817</v>
-      </c>
-      <c r="P20" s="11" t="n">
-        <v>0.6938657955501579</v>
-      </c>
-      <c r="Q20" s="7" t="n">
+      <c r="P20" s="10" t="n">
+        <v>42.66300973019838</v>
+      </c>
+      <c r="Q20" s="9" t="n">
+        <v>42663.00973019838</v>
+      </c>
+      <c r="R20" s="11" t="n">
+        <v>0.6879688919299324</v>
+      </c>
+      <c r="S20" s="7" t="n">
         <v>107</v>
       </c>
-      <c r="R20" s="12" t="n">
-        <v>-8170.034528261829</v>
-      </c>
-      <c r="S20" s="13" t="n">
-        <v>-0.1583340024856944</v>
-      </c>
-      <c r="T20" s="10" t="n">
+      <c r="T20" s="12" t="n">
+        <v>-8936.990269801616</v>
+      </c>
+      <c r="U20" s="13" t="n">
+        <v>-0.1731974858488686</v>
+      </c>
+      <c r="V20" s="10" t="n">
         <v>77.40000000000001</v>
       </c>
-      <c r="U20" s="14" t="n">
-        <v>0.7821796347125273</v>
-      </c>
-      <c r="V20" s="7" t="n">
+      <c r="W20" s="14" t="n">
+        <v>0.8142179956238192</v>
+      </c>
+      <c r="X20" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="W20" s="8" t="inlineStr">
+      <c r="Y20" s="8" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="X20" s="7" t="n">
+      <c r="Z20" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="Y20" s="8" t="inlineStr">
+      <c r="AA20" s="8" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1081,54 +1099,60 @@
       <c r="I21" s="17" t="n">
         <v>55410</v>
       </c>
-      <c r="J21" s="19" t="n">
+      <c r="J21" s="17" t="n">
+        <v>107010</v>
+      </c>
+      <c r="K21" s="17" t="n">
+        <v>106347.2485310492</v>
+      </c>
+      <c r="L21" s="19" t="n">
         <v>0.8</v>
       </c>
-      <c r="K21" s="15" t="n">
+      <c r="M21" s="15" t="n">
         <v>114</v>
       </c>
-      <c r="L21" s="17" t="n">
+      <c r="N21" s="17" t="n">
         <v>685</v>
       </c>
-      <c r="M21" s="17" t="n">
+      <c r="O21" s="17" t="n">
         <v>640</v>
       </c>
-      <c r="N21" s="18" t="n">
-        <v>47.0005424991154</v>
-      </c>
-      <c r="O21" s="17" t="n">
-        <v>47000.5424991154</v>
-      </c>
-      <c r="P21" s="19" t="n">
-        <v>0.7573043030830136</v>
-      </c>
-      <c r="Q21" s="15" t="n">
+      <c r="P21" s="18" t="n">
+        <v>46.1631346425541</v>
+      </c>
+      <c r="Q21" s="17" t="n">
+        <v>46163.1346425541</v>
+      </c>
+      <c r="R21" s="19" t="n">
+        <v>0.7514615997336538</v>
+      </c>
+      <c r="S21" s="15" t="n">
         <v>87</v>
       </c>
-      <c r="R21" s="12" t="n">
-        <v>-8409.4575008846</v>
-      </c>
-      <c r="S21" s="13" t="n">
-        <v>-0.1517678668270096</v>
-      </c>
-      <c r="T21" s="18" t="n">
+      <c r="T21" s="12" t="n">
+        <v>-9246.865357445902</v>
+      </c>
+      <c r="U21" s="13" t="n">
+        <v>-0.1668808041408752</v>
+      </c>
+      <c r="V21" s="18" t="n">
         <v>83.11499999999999</v>
       </c>
-      <c r="U21" s="20" t="n">
-        <v>0.7683838436878534</v>
-      </c>
-      <c r="V21" s="15" t="n">
+      <c r="W21" s="20" t="n">
+        <v>0.8004626558306318</v>
+      </c>
+      <c r="X21" s="15" t="n">
         <v>19</v>
       </c>
-      <c r="W21" s="16" t="inlineStr">
+      <c r="Y21" s="16" t="inlineStr">
         <is>
           <t>2026-04-29</t>
         </is>
       </c>
-      <c r="X21" s="15" t="n">
+      <c r="Z21" s="15" t="n">
         <v>41</v>
       </c>
-      <c r="Y21" s="16" t="inlineStr">
+      <c r="AA21" s="16" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1170,54 +1194,60 @@
       <c r="I22" s="9" t="n">
         <v>49700</v>
       </c>
-      <c r="J22" s="11" t="n">
+      <c r="J22" s="9" t="n">
+        <v>156710</v>
+      </c>
+      <c r="K22" s="9" t="n">
+        <v>164826.777974312</v>
+      </c>
+      <c r="L22" s="11" t="n">
         <v>0.76</v>
       </c>
-      <c r="K22" s="7" t="n">
+      <c r="M22" s="7" t="n">
         <v>98</v>
       </c>
-      <c r="L22" s="9" t="n">
+      <c r="N22" s="9" t="n">
         <v>684</v>
       </c>
-      <c r="M22" s="9" t="n">
+      <c r="O22" s="9" t="n">
         <v>640</v>
       </c>
-      <c r="N22" s="10" t="n">
-        <v>41.02663411338949</v>
-      </c>
-      <c r="O22" s="9" t="n">
-        <v>41026.63411338949</v>
-      </c>
-      <c r="P22" s="11" t="n">
-        <v>0.7380255638238143</v>
-      </c>
-      <c r="Q22" s="7" t="n">
+      <c r="P22" s="10" t="n">
+        <v>40.21106835529127</v>
+      </c>
+      <c r="Q22" s="9" t="n">
+        <v>40211.06835529127</v>
+      </c>
+      <c r="R22" s="11" t="n">
+        <v>0.731385012108221</v>
+      </c>
+      <c r="S22" s="7" t="n">
         <v>73</v>
       </c>
-      <c r="R22" s="12" t="n">
-        <v>-8673.365886610511</v>
-      </c>
-      <c r="S22" s="13" t="n">
-        <v>-0.1745144041571531</v>
-      </c>
-      <c r="T22" s="10" t="n">
+      <c r="T22" s="12" t="n">
+        <v>-9488.931644708726</v>
+      </c>
+      <c r="U22" s="13" t="n">
+        <v>-0.1909241779619463</v>
+      </c>
+      <c r="V22" s="10" t="n">
         <v>74.55000000000001</v>
       </c>
-      <c r="U22" s="14" t="n">
-        <v>0.8171122640467794</v>
-      </c>
-      <c r="V22" s="7" t="n">
+      <c r="W22" s="14" t="n">
+        <v>0.8539671550455128</v>
+      </c>
+      <c r="X22" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="W22" s="8" t="inlineStr">
+      <c r="Y22" s="8" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="X22" s="7" t="n">
+      <c r="Z22" s="7" t="n">
         <v>43</v>
       </c>
-      <c r="Y22" s="8" t="inlineStr">
+      <c r="AA22" s="8" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1259,54 +1289,60 @@
       <c r="I23" s="17" t="n">
         <v>51760</v>
       </c>
-      <c r="J23" s="19" t="n">
+      <c r="J23" s="17" t="n">
+        <v>208470</v>
+      </c>
+      <c r="K23" s="17" t="n">
+        <v>195947.4117740678</v>
+      </c>
+      <c r="L23" s="19" t="n">
         <v>0.78</v>
       </c>
-      <c r="K23" s="15" t="n">
+      <c r="M23" s="15" t="n">
         <v>119</v>
       </c>
-      <c r="L23" s="17" t="n">
+      <c r="N23" s="17" t="n">
         <v>688</v>
       </c>
-      <c r="M23" s="17" t="n">
+      <c r="O23" s="17" t="n">
         <v>641</v>
       </c>
-      <c r="N23" s="18" t="n">
-        <v>46.75090095676438</v>
-      </c>
-      <c r="O23" s="17" t="n">
-        <v>46750.90095676438</v>
-      </c>
-      <c r="P23" s="19" t="n">
-        <v>0.7206816059322184</v>
-      </c>
-      <c r="Q23" s="15" t="n">
+      <c r="P23" s="18" t="n">
+        <v>45.95404353893122</v>
+      </c>
+      <c r="Q23" s="17" t="n">
+        <v>45954.04353893122</v>
+      </c>
+      <c r="R23" s="19" t="n">
+        <v>0.7150268961679802</v>
+      </c>
+      <c r="S23" s="15" t="n">
         <v>107</v>
       </c>
-      <c r="R23" s="12" t="n">
-        <v>-5009.099043235619</v>
-      </c>
-      <c r="S23" s="13" t="n">
-        <v>-0.09677548383376378</v>
-      </c>
-      <c r="T23" s="18" t="n">
+      <c r="T23" s="12" t="n">
+        <v>-5805.956461068781</v>
+      </c>
+      <c r="U23" s="13" t="n">
+        <v>-0.1121707198815453</v>
+      </c>
+      <c r="V23" s="18" t="n">
         <v>77.64</v>
       </c>
-      <c r="U23" s="20" t="n">
-        <v>0.6607166580982495</v>
-      </c>
-      <c r="V23" s="15" t="n">
+      <c r="W23" s="20" t="n">
+        <v>0.6895140018358812</v>
+      </c>
+      <c r="X23" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="W23" s="16" t="inlineStr">
+      <c r="Y23" s="16" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="X23" s="15" t="n">
+      <c r="Z23" s="15" t="n">
         <v>52</v>
       </c>
-      <c r="Y23" s="16" t="inlineStr">
+      <c r="AA23" s="16" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1348,54 +1384,60 @@
       <c r="I24" s="9" t="n">
         <v>35840.00000000001</v>
       </c>
-      <c r="J24" s="11" t="n">
+      <c r="J24" s="9" t="n">
+        <v>244310</v>
+      </c>
+      <c r="K24" s="9" t="n">
+        <v>209201.577927858</v>
+      </c>
+      <c r="L24" s="11" t="n">
         <v>0.8</v>
       </c>
-      <c r="K24" s="7" t="n">
+      <c r="M24" s="7" t="n">
         <v>107</v>
       </c>
-      <c r="L24" s="9" t="n">
+      <c r="N24" s="9" t="n">
         <v>681.5</v>
       </c>
-      <c r="M24" s="9" t="n">
+      <c r="O24" s="9" t="n">
         <v>653</v>
       </c>
-      <c r="N24" s="10" t="n">
-        <v>69.36958909223097</v>
-      </c>
-      <c r="O24" s="9" t="n">
-        <v>34684.79454611548</v>
-      </c>
-      <c r="P24" s="11" t="n">
-        <v>0.8567727046411613</v>
-      </c>
-      <c r="Q24" s="7" t="n">
+      <c r="P24" s="10" t="n">
+        <v>68.42064332176614</v>
+      </c>
+      <c r="Q24" s="9" t="n">
+        <v>34210.32166088307</v>
+      </c>
+      <c r="R24" s="11" t="n">
+        <v>0.8529557469322286</v>
+      </c>
+      <c r="S24" s="7" t="n">
         <v>107</v>
       </c>
-      <c r="R24" s="12" t="n">
-        <v>-1155.205453884526</v>
-      </c>
-      <c r="S24" s="13" t="n">
-        <v>-0.03223229503026004</v>
-      </c>
-      <c r="T24" s="10" t="n">
+      <c r="T24" s="12" t="n">
+        <v>-1629.678339116937</v>
+      </c>
+      <c r="U24" s="13" t="n">
+        <v>-0.04547093580125383</v>
+      </c>
+      <c r="V24" s="10" t="n">
         <v>107.52</v>
       </c>
-      <c r="U24" s="14" t="n">
-        <v>0.549958726972504</v>
-      </c>
-      <c r="V24" s="7" t="n">
+      <c r="W24" s="14" t="n">
+        <v>0.5714555546395381</v>
+      </c>
+      <c r="X24" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="W24" s="8" t="inlineStr">
+      <c r="Y24" s="8" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="X24" s="7" t="n">
+      <c r="Z24" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="Y24" s="8" t="inlineStr">
+      <c r="AA24" s="8" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1437,54 +1479,60 @@
       <c r="I25" s="17" t="n">
         <v>35735</v>
       </c>
-      <c r="J25" s="19" t="n">
+      <c r="J25" s="17" t="n">
+        <v>280045</v>
+      </c>
+      <c r="K25" s="17" t="n">
+        <v>240587.2805939111</v>
+      </c>
+      <c r="L25" s="19" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="K25" s="15" t="n">
+      <c r="M25" s="15" t="n">
         <v>107</v>
       </c>
-      <c r="L25" s="17" t="n">
+      <c r="N25" s="17" t="n">
         <v>602.8</v>
       </c>
-      <c r="M25" s="17" t="n">
+      <c r="O25" s="17" t="n">
         <v>587</v>
       </c>
-      <c r="N25" s="18" t="n">
-        <v>63.73747329690349</v>
-      </c>
-      <c r="O25" s="17" t="n">
-        <v>31868.73664845174</v>
-      </c>
-      <c r="P25" s="19" t="n">
-        <v>0.8684766795783126</v>
-      </c>
-      <c r="Q25" s="15" t="n">
+      <c r="P25" s="18" t="n">
+        <v>62.77140533210604</v>
+      </c>
+      <c r="Q25" s="17" t="n">
+        <v>31385.70266605302</v>
+      </c>
+      <c r="R25" s="19" t="n">
+        <v>0.8643801683287227</v>
+      </c>
+      <c r="S25" s="15" t="n">
         <v>107</v>
       </c>
-      <c r="R25" s="12" t="n">
-        <v>-3866.263351548256</v>
-      </c>
-      <c r="S25" s="13" t="n">
-        <v>-0.1081926221225201</v>
-      </c>
-      <c r="T25" s="18" t="n">
+      <c r="T25" s="12" t="n">
+        <v>-4349.297333946979</v>
+      </c>
+      <c r="U25" s="13" t="n">
+        <v>-0.1217097337049665</v>
+      </c>
+      <c r="V25" s="18" t="n">
         <v>107.205</v>
       </c>
-      <c r="U25" s="20" t="n">
-        <v>0.6819775628791401</v>
-      </c>
-      <c r="V25" s="15" t="n">
+      <c r="W25" s="20" t="n">
+        <v>0.7078636272807366</v>
+      </c>
+      <c r="X25" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="W25" s="16" t="inlineStr">
+      <c r="Y25" s="16" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="X25" s="15" t="n">
+      <c r="Z25" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="Y25" s="16" t="inlineStr">
+      <c r="AA25" s="16" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1534,7 +1582,7 @@
         </is>
       </c>
       <c r="B31" s="23" t="n">
-        <v>244761.5742355747</v>
+        <v>240587.2805939111</v>
       </c>
     </row>
     <row r="32">
@@ -1544,7 +1592,7 @@
         </is>
       </c>
       <c r="B32" s="24" t="n">
-        <v>-35283.42576442534</v>
+        <v>-39457.71940608893</v>
       </c>
     </row>
     <row r="33">
@@ -1554,7 +1602,7 @@
         </is>
       </c>
       <c r="B33" s="25" t="n">
-        <v>-0.125991986160886</v>
+        <v>-0.1408977821638984</v>
       </c>
     </row>
     <row r="34">
@@ -1564,7 +1612,7 @@
         </is>
       </c>
       <c r="B34" s="26" t="n">
-        <v>3772.501960498941</v>
+        <v>3744.510357570263</v>
       </c>
     </row>
     <row r="35">
@@ -1574,7 +1622,7 @@
         </is>
       </c>
       <c r="B35" s="26" t="n">
-        <v>3772</v>
+        <v>3744</v>
       </c>
     </row>
     <row r="37">
@@ -1633,7 +1681,7 @@
         </is>
       </c>
       <c r="B39" s="9" t="n">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
@@ -1644,16 +1692,16 @@
         <v>108</v>
       </c>
       <c r="E39" s="11" t="n">
-        <v>0.7992885155618079</v>
+        <v>0.7984165368656055</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>72.40790436698552</v>
+        <v>72.36694565971817</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>72407.90436698552</v>
+        <v>72366.94565971817</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>36203.95218349276</v>
+        <v>36183.47282985909</v>
       </c>
     </row>
     <row r="40">
@@ -1663,7 +1711,7 @@
         </is>
       </c>
       <c r="B40" s="9" t="n">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
@@ -1674,22 +1722,21 @@
         <v>108</v>
       </c>
       <c r="E40" s="11" t="n">
-        <v>0.8018704887886536</v>
+        <v>0.8009709579873669</v>
       </c>
       <c r="F40" s="10" t="n">
-        <v>64.52805096752604</v>
+        <v>64.47162167597742</v>
       </c>
       <c r="G40" s="9" t="n">
-        <v>64528.05096752604</v>
+        <v>64471.62167597743</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>32264.02548376302</v>
+        <v>32235.81083798871</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="B12:F12"/>
-    <mergeCell ref="A2:Y2"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B16:F16"/>
@@ -1697,15 +1744,16 @@
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B5:F5"/>
-    <mergeCell ref="A1:Y1"/>
+    <mergeCell ref="A2:AA2"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="A18:V18"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="B8:F8"/>
+    <mergeCell ref="A27:H27"/>
     <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A1:AA1"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B13:F13"/>
+    <mergeCell ref="A18:X18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1761,7 +1809,7 @@
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
         <is>
-          <t>Last Updated: 2026-03-03 13:57:13  |  SPY: $681.09  |  QQQ: $602.48  |  PAPER TRADING - NOT REAL MONEY</t>
+          <t>Last Updated: 2026-03-03 14:12:15  |  SPY: $679.98  |  QQQ: $601.36  |  PAPER TRADING - NOT REAL MONEY</t>
         </is>
       </c>
     </row>
@@ -2377,25 +2425,25 @@
         <v>686.8</v>
       </c>
       <c r="V23" s="10" t="n">
-        <v>681.0900268554688</v>
+        <v>679.97998046875</v>
       </c>
       <c r="W23" s="38" t="n">
         <v>19.92000007629395</v>
       </c>
       <c r="X23" s="38" t="n">
-        <v>22.71999931335449</v>
+        <v>22.80999946594238</v>
       </c>
       <c r="Y23" s="14" t="n">
         <v>0.1659804310259251</v>
       </c>
       <c r="Z23" s="14" t="n">
-        <v>0.2380339339689771</v>
+        <v>0.240349943978385</v>
       </c>
       <c r="AA23" s="10" t="n">
         <v>648.5776251220703</v>
       </c>
       <c r="AB23" s="10" t="n">
-        <v>652.7582373046876</v>
+        <v>652.752537536621</v>
       </c>
       <c r="AC23" s="8" t="inlineStr">
         <is>
@@ -2476,25 +2524,25 @@
         <v>606.785</v>
       </c>
       <c r="V24" s="10" t="n">
-        <v>602.47998046875</v>
+        <v>601.364990234375</v>
       </c>
       <c r="W24" s="38" t="n">
         <v>20.29000091552734</v>
       </c>
       <c r="X24" s="38" t="n">
-        <v>22.71999931335449</v>
+        <v>22.80999946594238</v>
       </c>
       <c r="Y24" s="14" t="n">
         <v>0.175501810962665</v>
       </c>
       <c r="Z24" s="14" t="n">
-        <v>0.2380339339689771</v>
+        <v>0.240349943978385</v>
       </c>
       <c r="AA24" s="10" t="n">
         <v>582.6986384582519</v>
       </c>
       <c r="AB24" s="10" t="n">
-        <v>586.6202792358398</v>
+        <v>586.6145758056641</v>
       </c>
       <c r="AC24" s="8" t="inlineStr">
         <is>
@@ -2690,25 +2738,25 @@
         <v>687.6799999999999</v>
       </c>
       <c r="V26" s="10" t="n">
-        <v>681.0900268554688</v>
+        <v>679.97998046875</v>
       </c>
       <c r="W26" s="38" t="n">
         <v>19.94000053405762</v>
       </c>
       <c r="X26" s="38" t="n">
-        <v>22.71999931335449</v>
+        <v>22.80999946594238</v>
       </c>
       <c r="Y26" s="14" t="n">
         <v>0.1664951108241417</v>
       </c>
       <c r="Z26" s="14" t="n">
-        <v>0.2380339339689771</v>
+        <v>0.240349943978385</v>
       </c>
       <c r="AA26" s="10" t="n">
         <v>651.1943740844727</v>
       </c>
       <c r="AB26" s="10" t="n">
-        <v>652.7582373046876</v>
+        <v>652.752537536621</v>
       </c>
       <c r="AC26" s="8" t="inlineStr">
         <is>
@@ -2789,25 +2837,25 @@
         <v>257.93</v>
       </c>
       <c r="V27" s="10" t="n">
-        <v>260.625</v>
+        <v>260.0350036621094</v>
       </c>
       <c r="W27" s="38" t="n">
         <v>24.10000038146973</v>
       </c>
       <c r="X27" s="38" t="n">
-        <v>22.71999931335449</v>
+        <v>22.80999946594238</v>
       </c>
       <c r="Y27" s="14" t="n">
         <v>0.2735460547248535</v>
       </c>
       <c r="Z27" s="14" t="n">
-        <v>0.2380339339689771</v>
+        <v>0.240349943978385</v>
       </c>
       <c r="AA27" s="10" t="n">
         <v>237.4489370727539</v>
       </c>
       <c r="AB27" s="10" t="n">
-        <v>237.4623371887207</v>
+        <v>237.4594620513916</v>
       </c>
       <c r="AC27" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add TSLA bear put spread + UPRO DD25/Cool40 sheets to position tracker
- Sheet 3: TSLA $300/$250 bear put debit spread with Greeks (ThetaData + BS fallback)
- Sheet 4: UPRO 1000-share long position with DD25%/Cool40 drawdown monitoring
- New helpers: bs_put_greeks, get_thetadata_greeks, get_tsla_iv_from_yfinance

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Strategies/80-Delta Call Strategy/position_tracker.xlsx
+++ b/Strategies/80-Delta Call Strategy/position_tracker.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="80-Delta Calls" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCS Paper Trades" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TSLA Bear Put Spread" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UPRO DD25-Cool40" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,12 +19,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="0.1%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,8 +91,38 @@
       <color rgb="00006100"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="007B2020"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="007B2020"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="001B5E20"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B5E20"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -143,8 +177,32 @@
         <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007B2020"/>
+        <bgColor rgb="007B2020"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A03030"/>
+        <bgColor rgb="00A03030"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B5E20"/>
+        <bgColor rgb="001B5E20"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E7D32"/>
+        <bgColor rgb="002E7D32"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -158,11 +216,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -273,6 +359,59 @@
     </xf>
     <xf numFmtId="165" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -639,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA40"/>
+  <dimension ref="A1:AA41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -681,1079 +820,1087 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last Updated: 2026-03-03 14:12:14  |  SPY: $679.98  |  QQQ: $601.36</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+          <t>Last Updated: 2026-03-10 20:16:17  |  SPY: $677.18  |  QQQ: $607.77</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SPY SMA200: $655.08 (+3.4%)  |  QQQ SMA200: $588.86 (+3.2%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Strategy Criteria</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Entry Rules</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Signal</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>SPY &gt; 200-day SMA</t>
-        </is>
-      </c>
+      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Delta</t>
+          <t xml:space="preserve">  Signal</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>70-80 delta at entry</t>
+          <t>SPY &gt; 200-day SMA</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DTE</t>
+          <t xml:space="preserve">  Delta</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>90-150 days to expiration</t>
+          <t>70-80 delta at entry</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">  DTE</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>90-150 days to expiration</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Frequency</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Monthly only (standard expiry)</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Exit Rules</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Profit Target</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>+50% from entry price</t>
-        </is>
-      </c>
+      <c r="B11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Max Hold</t>
+          <t xml:space="preserve">  Profit Target</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>60 trading days</t>
+          <t>+50% from entry price</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SMA Breach</t>
+          <t xml:space="preserve">  Max Hold</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Optional: exit if SPY &gt;2% below SMA200</t>
+          <t>60 trading days</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">  SMA Breach</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Optional: exit if SPY &gt;2% below SMA200</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Stop Loss</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>None (per backtest results)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="B16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Delta Cap</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Monitor total delta exposure (not a hard limit)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Open Positions</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Trade #</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Entry Date</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Symbol</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>Strike</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>Expiration</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>Entry Price</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>Total Cost</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>Capital Invested</t>
         </is>
       </c>
-      <c r="K19" s="6" t="inlineStr">
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>Market Value</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr">
         <is>
           <t>Delta@Entry</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
+      <c r="M20" s="6" t="inlineStr">
         <is>
           <t>DTE@Entry</t>
         </is>
       </c>
-      <c r="N19" s="6" t="inlineStr">
+      <c r="N20" s="6" t="inlineStr">
         <is>
           <t>SPY@Entry</t>
         </is>
       </c>
-      <c r="O19" s="6" t="inlineStr">
+      <c r="O20" s="6" t="inlineStr">
         <is>
           <t>SMA200@Entry</t>
         </is>
       </c>
-      <c r="P19" s="6" t="inlineStr">
+      <c r="P20" s="6" t="inlineStr">
         <is>
           <t>Current Price</t>
         </is>
       </c>
-      <c r="Q19" s="6" t="inlineStr">
+      <c r="Q20" s="6" t="inlineStr">
         <is>
           <t>Current Value</t>
         </is>
       </c>
-      <c r="R19" s="6" t="inlineStr">
+      <c r="R20" s="6" t="inlineStr">
         <is>
           <t>Cur Delta</t>
         </is>
       </c>
-      <c r="S19" s="6" t="inlineStr">
+      <c r="S20" s="6" t="inlineStr">
         <is>
           <t>Cur DTE</t>
         </is>
       </c>
-      <c r="T19" s="6" t="inlineStr">
+      <c r="T20" s="6" t="inlineStr">
         <is>
           <t>Unreal P&amp;L ($)</t>
         </is>
       </c>
-      <c r="U19" s="6" t="inlineStr">
+      <c r="U20" s="6" t="inlineStr">
         <is>
           <t>Unreal P&amp;L (%)</t>
         </is>
       </c>
-      <c r="V19" s="6" t="inlineStr">
+      <c r="V20" s="6" t="inlineStr">
         <is>
           <t>Target Price</t>
         </is>
       </c>
-      <c r="W19" s="6" t="inlineStr">
+      <c r="W20" s="6" t="inlineStr">
         <is>
           <t>% To Target</t>
         </is>
       </c>
-      <c r="X19" s="6" t="inlineStr">
+      <c r="X20" s="6" t="inlineStr">
         <is>
           <t>Days Held</t>
         </is>
       </c>
-      <c r="Y19" s="6" t="inlineStr">
+      <c r="Y20" s="6" t="inlineStr">
         <is>
           <t>Max Hold Date</t>
         </is>
       </c>
-      <c r="Z19" s="6" t="inlineStr">
+      <c r="Z20" s="6" t="inlineStr">
         <is>
           <t>Days Remaining</t>
         </is>
       </c>
-      <c r="AA19" s="6" t="inlineStr">
+      <c r="AA20" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="7" t="n">
+    <row r="21">
+      <c r="A21" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>2026-02-03</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="D21" s="9" t="n">
         <v>660</v>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>CALL</t>
         </is>
       </c>
-      <c r="G20" s="7" t="n">
+      <c r="G21" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="H20" s="10" t="n">
+      <c r="H21" s="10" t="n">
         <v>51.6</v>
       </c>
-      <c r="I20" s="9" t="n">
+      <c r="I21" s="9" t="n">
         <v>51600</v>
       </c>
-      <c r="J20" s="9" t="n">
+      <c r="J21" s="9" t="n">
         <v>51600</v>
       </c>
-      <c r="K20" s="9" t="n">
+      <c r="K21" s="9" t="n">
         <v>53761.53242392735</v>
       </c>
-      <c r="L20" s="11" t="n">
+      <c r="L21" s="11" t="n">
         <v>0.74</v>
       </c>
-      <c r="M20" s="7" t="n">
+      <c r="M21" s="7" t="n">
         <v>135</v>
       </c>
-      <c r="N20" s="9" t="n">
+      <c r="N21" s="9" t="n">
         <v>687</v>
       </c>
-      <c r="O20" s="9" t="n">
+      <c r="O21" s="9" t="n">
         <v>640</v>
       </c>
-      <c r="P20" s="10" t="n">
-        <v>42.66300973019838</v>
-      </c>
-      <c r="Q20" s="9" t="n">
-        <v>42663.00973019838</v>
-      </c>
-      <c r="R20" s="11" t="n">
-        <v>0.6879688919299324</v>
-      </c>
-      <c r="S20" s="7" t="n">
+      <c r="P21" s="10" t="n">
+        <v>39.6072213876563</v>
+      </c>
+      <c r="Q21" s="9" t="n">
+        <v>39607.2213876563</v>
+      </c>
+      <c r="R21" s="11" t="n">
+        <v>0.6739013349292748</v>
+      </c>
+      <c r="S21" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="T21" s="12" t="n">
+        <v>-11992.7786123437</v>
+      </c>
+      <c r="U21" s="13" t="n">
+        <v>-0.2324181901616997</v>
+      </c>
+      <c r="V21" s="10" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="W21" s="14" t="n">
+        <v>0.9541890919952779</v>
+      </c>
+      <c r="X21" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y21" s="8" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="Z21" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="AA21" s="8" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="n">
+        <v>650</v>
+      </c>
+      <c r="E22" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="H22" s="18" t="n">
+        <v>55.41</v>
+      </c>
+      <c r="I22" s="17" t="n">
+        <v>55410</v>
+      </c>
+      <c r="J22" s="17" t="n">
+        <v>107010</v>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v>106347.2485310492</v>
+      </c>
+      <c r="L22" s="19" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="M22" s="15" t="n">
+        <v>114</v>
+      </c>
+      <c r="N22" s="17" t="n">
+        <v>685</v>
+      </c>
+      <c r="O22" s="17" t="n">
+        <v>640</v>
+      </c>
+      <c r="P22" s="18" t="n">
+        <v>42.89079616610218</v>
+      </c>
+      <c r="Q22" s="17" t="n">
+        <v>42890.79616610217</v>
+      </c>
+      <c r="R22" s="19" t="n">
+        <v>0.7406307270636951</v>
+      </c>
+      <c r="S22" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="T22" s="12" t="n">
+        <v>-12519.20383389783</v>
+      </c>
+      <c r="U22" s="13" t="n">
+        <v>-0.2259376255892045</v>
+      </c>
+      <c r="V22" s="18" t="n">
+        <v>83.11499999999999</v>
+      </c>
+      <c r="W22" s="20" t="n">
+        <v>0.9378283321699716</v>
+      </c>
+      <c r="X22" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="Y22" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="Z22" s="15" t="n">
+        <v>36</v>
+      </c>
+      <c r="AA22" s="16" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>655</v>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="I23" s="9" t="n">
+        <v>49700</v>
+      </c>
+      <c r="J23" s="9" t="n">
+        <v>156710</v>
+      </c>
+      <c r="K23" s="9" t="n">
+        <v>164826.777974312</v>
+      </c>
+      <c r="L23" s="11" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="M23" s="7" t="n">
+        <v>98</v>
+      </c>
+      <c r="N23" s="9" t="n">
+        <v>684</v>
+      </c>
+      <c r="O23" s="9" t="n">
+        <v>640</v>
+      </c>
+      <c r="P23" s="10" t="n">
+        <v>36.8934173771782</v>
+      </c>
+      <c r="Q23" s="9" t="n">
+        <v>36893.41737717819</v>
+      </c>
+      <c r="R23" s="11" t="n">
+        <v>0.7189281090771118</v>
+      </c>
+      <c r="S23" s="7" t="n">
+        <v>66</v>
+      </c>
+      <c r="T23" s="12" t="n">
+        <v>-12806.58262282181</v>
+      </c>
+      <c r="U23" s="13" t="n">
+        <v>-0.2576777187690504</v>
+      </c>
+      <c r="V23" s="10" t="n">
+        <v>74.55000000000001</v>
+      </c>
+      <c r="W23" s="14" t="n">
+        <v>1.020685675112214</v>
+      </c>
+      <c r="X23" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="Y23" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="Z23" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="AA23" s="8" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="n">
+        <v>655</v>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="H24" s="18" t="n">
+        <v>51.76</v>
+      </c>
+      <c r="I24" s="17" t="n">
+        <v>51760</v>
+      </c>
+      <c r="J24" s="17" t="n">
+        <v>208470</v>
+      </c>
+      <c r="K24" s="17" t="n">
+        <v>195947.4117740678</v>
+      </c>
+      <c r="L24" s="19" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="M24" s="15" t="n">
+        <v>119</v>
+      </c>
+      <c r="N24" s="17" t="n">
+        <v>688</v>
+      </c>
+      <c r="O24" s="17" t="n">
+        <v>641</v>
+      </c>
+      <c r="P24" s="18" t="n">
+        <v>42.83815801513327</v>
+      </c>
+      <c r="Q24" s="17" t="n">
+        <v>42838.15801513327</v>
+      </c>
+      <c r="R24" s="19" t="n">
+        <v>0.7024381907695142</v>
+      </c>
+      <c r="S24" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="T24" s="12" t="n">
+        <v>-8921.841984866725</v>
+      </c>
+      <c r="U24" s="13" t="n">
+        <v>-0.1723694355654313</v>
+      </c>
+      <c r="V24" s="18" t="n">
+        <v>77.64</v>
+      </c>
+      <c r="W24" s="20" t="n">
+        <v>0.8124028575778728</v>
+      </c>
+      <c r="X24" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="Y24" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="Z24" s="15" t="n">
+        <v>47</v>
+      </c>
+      <c r="AA24" s="16" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>625</v>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H25" s="10" t="n">
+        <v>71.68000000000001</v>
+      </c>
+      <c r="I25" s="9" t="n">
+        <v>35840.00000000001</v>
+      </c>
+      <c r="J25" s="9" t="n">
+        <v>244310</v>
+      </c>
+      <c r="K25" s="9" t="n">
+        <v>210362.4505010633</v>
+      </c>
+      <c r="L25" s="11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="M25" s="7" t="n">
         <v>107</v>
       </c>
-      <c r="T20" s="12" t="n">
-        <v>-8936.990269801616</v>
-      </c>
-      <c r="U20" s="13" t="n">
-        <v>-0.1731974858488686</v>
-      </c>
-      <c r="V20" s="10" t="n">
-        <v>77.40000000000001</v>
-      </c>
-      <c r="W20" s="14" t="n">
-        <v>0.8142179956238192</v>
-      </c>
-      <c r="X20" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="Y20" s="8" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-      <c r="Z20" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="AA20" s="8" t="inlineStr">
+      <c r="N25" s="9" t="n">
+        <v>681.5</v>
+      </c>
+      <c r="O25" s="9" t="n">
+        <v>653</v>
+      </c>
+      <c r="P25" s="10" t="n">
+        <v>65.0868710932462</v>
+      </c>
+      <c r="Q25" s="9" t="n">
+        <v>32543.4355466231</v>
+      </c>
+      <c r="R25" s="11" t="n">
+        <v>0.8482701381105086</v>
+      </c>
+      <c r="S25" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="T25" s="12" t="n">
+        <v>-3296.564453376908</v>
+      </c>
+      <c r="U25" s="13" t="n">
+        <v>-0.09198003497145368</v>
+      </c>
+      <c r="V25" s="10" t="n">
+        <v>107.52</v>
+      </c>
+      <c r="W25" s="14" t="n">
+        <v>0.6519460560020209</v>
+      </c>
+      <c r="X25" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y25" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="Z25" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="AA25" s="8" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="B21" s="16" t="inlineStr">
-        <is>
-          <t>2026-02-04</t>
-        </is>
-      </c>
-      <c r="C21" s="16" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D21" s="17" t="n">
-        <v>650</v>
-      </c>
-      <c r="E21" s="16" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="F21" s="16" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="n">
+        <v>550</v>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <t>CALL</t>
         </is>
       </c>
-      <c r="G21" s="15" t="n">
-        <v>10</v>
-      </c>
-      <c r="H21" s="18" t="n">
-        <v>55.41</v>
-      </c>
-      <c r="I21" s="17" t="n">
-        <v>55410</v>
-      </c>
-      <c r="J21" s="17" t="n">
-        <v>107010</v>
-      </c>
-      <c r="K21" s="17" t="n">
-        <v>106347.2485310492</v>
-      </c>
-      <c r="L21" s="19" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="M21" s="15" t="n">
-        <v>114</v>
-      </c>
-      <c r="N21" s="17" t="n">
-        <v>685</v>
-      </c>
-      <c r="O21" s="17" t="n">
-        <v>640</v>
-      </c>
-      <c r="P21" s="18" t="n">
-        <v>46.1631346425541</v>
-      </c>
-      <c r="Q21" s="17" t="n">
-        <v>46163.1346425541</v>
-      </c>
-      <c r="R21" s="19" t="n">
-        <v>0.7514615997336538</v>
-      </c>
-      <c r="S21" s="15" t="n">
-        <v>87</v>
-      </c>
-      <c r="T21" s="12" t="n">
-        <v>-9246.865357445902</v>
-      </c>
-      <c r="U21" s="13" t="n">
-        <v>-0.1668808041408752</v>
-      </c>
-      <c r="V21" s="18" t="n">
-        <v>83.11499999999999</v>
-      </c>
-      <c r="W21" s="20" t="n">
-        <v>0.8004626558306318</v>
-      </c>
-      <c r="X21" s="15" t="n">
-        <v>19</v>
-      </c>
-      <c r="Y21" s="16" t="inlineStr">
-        <is>
-          <t>2026-04-29</t>
-        </is>
-      </c>
-      <c r="Z21" s="15" t="n">
-        <v>41</v>
-      </c>
-      <c r="AA21" s="16" t="inlineStr">
+      <c r="G26" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="H26" s="18" t="n">
+        <v>71.47</v>
+      </c>
+      <c r="I26" s="17" t="n">
+        <v>35735</v>
+      </c>
+      <c r="J26" s="17" t="n">
+        <v>280045</v>
+      </c>
+      <c r="K26" s="17" t="n">
+        <v>241841.1285355787</v>
+      </c>
+      <c r="L26" s="19" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="M26" s="15" t="n">
+        <v>107</v>
+      </c>
+      <c r="N26" s="17" t="n">
+        <v>602.8</v>
+      </c>
+      <c r="O26" s="17" t="n">
+        <v>587</v>
+      </c>
+      <c r="P26" s="18" t="n">
+        <v>67.60096608682267</v>
+      </c>
+      <c r="Q26" s="17" t="n">
+        <v>33800.48304341133</v>
+      </c>
+      <c r="R26" s="19" t="n">
+        <v>0.8921530107565758</v>
+      </c>
+      <c r="S26" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="T26" s="12" t="n">
+        <v>-1934.516956588668</v>
+      </c>
+      <c r="U26" s="13" t="n">
+        <v>-0.05413507644014737</v>
+      </c>
+      <c r="V26" s="18" t="n">
+        <v>107.205</v>
+      </c>
+      <c r="W26" s="20" t="n">
+        <v>0.5858501173239486</v>
+      </c>
+      <c r="X26" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y26" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="Z26" s="15" t="n">
+        <v>55</v>
+      </c>
+      <c r="AA26" s="16" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>2026-02-06</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="n">
-        <v>655</v>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="H22" s="10" t="n">
-        <v>49.7</v>
-      </c>
-      <c r="I22" s="9" t="n">
-        <v>49700</v>
-      </c>
-      <c r="J22" s="9" t="n">
-        <v>156710</v>
-      </c>
-      <c r="K22" s="9" t="n">
-        <v>164826.777974312</v>
-      </c>
-      <c r="L22" s="11" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="M22" s="7" t="n">
-        <v>98</v>
-      </c>
-      <c r="N22" s="9" t="n">
-        <v>684</v>
-      </c>
-      <c r="O22" s="9" t="n">
-        <v>640</v>
-      </c>
-      <c r="P22" s="10" t="n">
-        <v>40.21106835529127</v>
-      </c>
-      <c r="Q22" s="9" t="n">
-        <v>40211.06835529127</v>
-      </c>
-      <c r="R22" s="11" t="n">
-        <v>0.731385012108221</v>
-      </c>
-      <c r="S22" s="7" t="n">
-        <v>73</v>
-      </c>
-      <c r="T22" s="12" t="n">
-        <v>-9488.931644708726</v>
-      </c>
-      <c r="U22" s="13" t="n">
-        <v>-0.1909241779619463</v>
-      </c>
-      <c r="V22" s="10" t="n">
-        <v>74.55000000000001</v>
-      </c>
-      <c r="W22" s="14" t="n">
-        <v>0.8539671550455128</v>
-      </c>
-      <c r="X22" s="7" t="n">
-        <v>17</v>
-      </c>
-      <c r="Y22" s="8" t="inlineStr">
-        <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="Z22" s="7" t="n">
-        <v>43</v>
-      </c>
-      <c r="AA22" s="8" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="B23" s="16" t="inlineStr">
-        <is>
-          <t>2026-02-19</t>
-        </is>
-      </c>
-      <c r="C23" s="16" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D23" s="17" t="n">
-        <v>655</v>
-      </c>
-      <c r="E23" s="16" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="G23" s="15" t="n">
-        <v>10</v>
-      </c>
-      <c r="H23" s="18" t="n">
-        <v>51.76</v>
-      </c>
-      <c r="I23" s="17" t="n">
-        <v>51760</v>
-      </c>
-      <c r="J23" s="17" t="n">
-        <v>208470</v>
-      </c>
-      <c r="K23" s="17" t="n">
-        <v>195947.4117740678</v>
-      </c>
-      <c r="L23" s="19" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="M23" s="15" t="n">
-        <v>119</v>
-      </c>
-      <c r="N23" s="17" t="n">
-        <v>688</v>
-      </c>
-      <c r="O23" s="17" t="n">
-        <v>641</v>
-      </c>
-      <c r="P23" s="18" t="n">
-        <v>45.95404353893122</v>
-      </c>
-      <c r="Q23" s="17" t="n">
-        <v>45954.04353893122</v>
-      </c>
-      <c r="R23" s="19" t="n">
-        <v>0.7150268961679802</v>
-      </c>
-      <c r="S23" s="15" t="n">
-        <v>107</v>
-      </c>
-      <c r="T23" s="12" t="n">
-        <v>-5805.956461068781</v>
-      </c>
-      <c r="U23" s="13" t="n">
-        <v>-0.1121707198815453</v>
-      </c>
-      <c r="V23" s="18" t="n">
-        <v>77.64</v>
-      </c>
-      <c r="W23" s="20" t="n">
-        <v>0.6895140018358812</v>
-      </c>
-      <c r="X23" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="Y23" s="16" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="Z23" s="15" t="n">
-        <v>52</v>
-      </c>
-      <c r="AA23" s="16" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>2026-03-03</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="n">
-        <v>625</v>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="H24" s="10" t="n">
-        <v>71.68000000000001</v>
-      </c>
-      <c r="I24" s="9" t="n">
-        <v>35840.00000000001</v>
-      </c>
-      <c r="J24" s="9" t="n">
-        <v>244310</v>
-      </c>
-      <c r="K24" s="9" t="n">
-        <v>209201.577927858</v>
-      </c>
-      <c r="L24" s="11" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="M24" s="7" t="n">
-        <v>107</v>
-      </c>
-      <c r="N24" s="9" t="n">
-        <v>681.5</v>
-      </c>
-      <c r="O24" s="9" t="n">
-        <v>653</v>
-      </c>
-      <c r="P24" s="10" t="n">
-        <v>68.42064332176614</v>
-      </c>
-      <c r="Q24" s="9" t="n">
-        <v>34210.32166088307</v>
-      </c>
-      <c r="R24" s="11" t="n">
-        <v>0.8529557469322286</v>
-      </c>
-      <c r="S24" s="7" t="n">
-        <v>107</v>
-      </c>
-      <c r="T24" s="12" t="n">
-        <v>-1629.678339116937</v>
-      </c>
-      <c r="U24" s="13" t="n">
-        <v>-0.04547093580125383</v>
-      </c>
-      <c r="V24" s="10" t="n">
-        <v>107.52</v>
-      </c>
-      <c r="W24" s="14" t="n">
-        <v>0.5714555546395381</v>
-      </c>
-      <c r="X24" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y24" s="8" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="Z24" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="AA24" s="8" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="B25" s="16" t="inlineStr">
-        <is>
-          <t>2026-03-03</t>
-        </is>
-      </c>
-      <c r="C25" s="16" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="D25" s="17" t="n">
-        <v>550</v>
-      </c>
-      <c r="E25" s="16" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="F25" s="16" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="G25" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="H25" s="18" t="n">
-        <v>71.47</v>
-      </c>
-      <c r="I25" s="17" t="n">
-        <v>35735</v>
-      </c>
-      <c r="J25" s="17" t="n">
-        <v>280045</v>
-      </c>
-      <c r="K25" s="17" t="n">
-        <v>240587.2805939111</v>
-      </c>
-      <c r="L25" s="19" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="M25" s="15" t="n">
-        <v>107</v>
-      </c>
-      <c r="N25" s="17" t="n">
-        <v>602.8</v>
-      </c>
-      <c r="O25" s="17" t="n">
-        <v>587</v>
-      </c>
-      <c r="P25" s="18" t="n">
-        <v>62.77140533210604</v>
-      </c>
-      <c r="Q25" s="17" t="n">
-        <v>31385.70266605302</v>
-      </c>
-      <c r="R25" s="19" t="n">
-        <v>0.8643801683287227</v>
-      </c>
-      <c r="S25" s="15" t="n">
-        <v>107</v>
-      </c>
-      <c r="T25" s="12" t="n">
-        <v>-4349.297333946979</v>
-      </c>
-      <c r="U25" s="13" t="n">
-        <v>-0.1217097337049665</v>
-      </c>
-      <c r="V25" s="18" t="n">
-        <v>107.205</v>
-      </c>
-      <c r="W25" s="20" t="n">
-        <v>0.7078636272807366</v>
-      </c>
-      <c r="X25" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y25" s="16" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="Z25" s="15" t="n">
-        <v>60</v>
-      </c>
-      <c r="AA25" s="16" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Portfolio Summary</t>
         </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="21" t="inlineStr">
-        <is>
-          <t>Open Positions</t>
-        </is>
-      </c>
-      <c r="B28" s="22" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="21" t="inlineStr">
         <is>
-          <t>Total Contracts</t>
+          <t>Open Positions</t>
         </is>
       </c>
       <c r="B29" s="22" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="21" t="inlineStr">
         <is>
-          <t>Total Cost Basis</t>
-        </is>
-      </c>
-      <c r="B30" s="23" t="n">
-        <v>280045</v>
+          <t>Total Contracts</t>
+        </is>
+      </c>
+      <c r="B30" s="22" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="21" t="inlineStr">
         <is>
-          <t>Total Current Value</t>
+          <t>Total Cost Basis</t>
         </is>
       </c>
       <c r="B31" s="23" t="n">
-        <v>240587.2805939111</v>
+        <v>280045</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="21" t="inlineStr">
         <is>
-          <t>Total Unrealized P&amp;L</t>
-        </is>
-      </c>
-      <c r="B32" s="24" t="n">
-        <v>-39457.71940608893</v>
+          <t>Total Current Value</t>
+        </is>
+      </c>
+      <c r="B32" s="23" t="n">
+        <v>228573.5115361044</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="21" t="inlineStr">
         <is>
-          <t>Total P&amp;L %</t>
-        </is>
-      </c>
-      <c r="B33" s="25" t="n">
-        <v>-0.1408977821638984</v>
+          <t>Total Unrealized P&amp;L</t>
+        </is>
+      </c>
+      <c r="B33" s="24" t="n">
+        <v>-51471.48846389563</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="21" t="inlineStr">
         <is>
-          <t>Total Delta Exposure</t>
-        </is>
-      </c>
-      <c r="B34" s="26" t="n">
-        <v>3744.510357570263</v>
+          <t>Total P&amp;L %</t>
+        </is>
+      </c>
+      <c r="B34" s="25" t="n">
+        <v>-0.1837972056772863</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="21" t="inlineStr">
         <is>
+          <t>Total Delta Exposure</t>
+        </is>
+      </c>
+      <c r="B35" s="26" t="n">
+        <v>3706.109936273138</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="21" t="inlineStr">
+        <is>
           <t>Equivalent SPY Shares</t>
         </is>
       </c>
-      <c r="B35" s="26" t="n">
-        <v>3744</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="B36" s="26" t="n">
+        <v>3706</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>Recommended Next Trades</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>Symbol</t>
         </is>
       </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>Strike</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>Expiration</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>DTE</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>Est Delta</t>
         </is>
       </c>
-      <c r="F38" s="6" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>Est Price</t>
         </is>
       </c>
-      <c r="G38" s="6" t="inlineStr">
+      <c r="G39" s="6" t="inlineStr">
         <is>
           <t>Cost (10 ct)</t>
         </is>
       </c>
-      <c r="H38" s="6" t="inlineStr">
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>Cost (5 ct)</t>
         </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="B39" s="9" t="n">
-        <v>626</v>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="E39" s="11" t="n">
-        <v>0.7984165368656055</v>
-      </c>
-      <c r="F39" s="10" t="n">
-        <v>72.36694565971817</v>
-      </c>
-      <c r="G39" s="9" t="n">
-        <v>72366.94565971817</v>
-      </c>
-      <c r="H39" s="9" t="n">
-        <v>36183.47282985909</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="n">
+        <v>614</v>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="n">
+        <v>129</v>
+      </c>
+      <c r="E40" s="11" t="n">
+        <v>0.8001781124678849</v>
+      </c>
+      <c r="F40" s="10" t="n">
+        <v>84.899162985239</v>
+      </c>
+      <c r="G40" s="9" t="n">
+        <v>84899.162985239</v>
+      </c>
+      <c r="H40" s="9" t="n">
+        <v>42449.5814926195</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="B40" s="9" t="n">
-        <v>553</v>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="E40" s="11" t="n">
-        <v>0.8009709579873669</v>
-      </c>
-      <c r="F40" s="10" t="n">
-        <v>64.47162167597742</v>
-      </c>
-      <c r="G40" s="9" t="n">
-        <v>64471.62167597743</v>
-      </c>
-      <c r="H40" s="9" t="n">
-        <v>32235.81083798871</v>
+      <c r="B41" s="9" t="n">
+        <v>551</v>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="n">
+        <v>129</v>
+      </c>
+      <c r="E41" s="11" t="n">
+        <v>0.8004037738276757</v>
+      </c>
+      <c r="F41" s="10" t="n">
+        <v>76.24616385754177</v>
+      </c>
+      <c r="G41" s="9" t="n">
+        <v>76246.16385754177</v>
+      </c>
+      <c r="H41" s="9" t="n">
+        <v>38123.08192877089</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B16:F16"/>
     <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="A3:AA3"/>
+    <mergeCell ref="A5:F5"/>
     <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B5:F5"/>
     <mergeCell ref="A2:AA2"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="A4:F4"/>
     <mergeCell ref="B8:F8"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="A19:X19"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A1:AA1"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="A18:X18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1809,7 +1956,7 @@
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
         <is>
-          <t>Last Updated: 2026-03-03 14:12:15  |  SPY: $679.98  |  QQQ: $601.36  |  PAPER TRADING - NOT REAL MONEY</t>
+          <t>Last Updated: 2026-03-10 20:16:17  |  SPY: $677.18  |  QQQ: $607.77  |  PAPER TRADING - NOT REAL MONEY</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2524,7 @@
         </is>
       </c>
       <c r="F23" s="8" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G23" s="10" t="n">
         <v>657</v>
@@ -2407,13 +2554,13 @@
         <v>9.92</v>
       </c>
       <c r="P23" s="10" t="n">
-        <v>4.024999999999999</v>
+        <v>4.38</v>
       </c>
       <c r="Q23" s="12" t="n">
-        <v>-3089.999999999999</v>
+        <v>-3800</v>
       </c>
       <c r="R23" s="13" t="n">
-        <v>-0.6229838709677418</v>
+        <v>-0.7661290322580645</v>
       </c>
       <c r="S23" s="9" t="n">
         <v>4960</v>
@@ -2425,25 +2572,25 @@
         <v>686.8</v>
       </c>
       <c r="V23" s="10" t="n">
-        <v>679.97998046875</v>
+        <v>677.1799926757812</v>
       </c>
       <c r="W23" s="38" t="n">
         <v>19.92000007629395</v>
       </c>
       <c r="X23" s="38" t="n">
-        <v>22.80999946594238</v>
+        <v>24.93000030517578</v>
       </c>
       <c r="Y23" s="14" t="n">
         <v>0.1659804310259251</v>
       </c>
       <c r="Z23" s="14" t="n">
-        <v>0.240349943978385</v>
+        <v>0.2949047755251742</v>
       </c>
       <c r="AA23" s="10" t="n">
         <v>648.5776251220703</v>
       </c>
       <c r="AB23" s="10" t="n">
-        <v>652.752537536621</v>
+        <v>655.0772604370118</v>
       </c>
       <c r="AC23" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2623,7 @@
         </is>
       </c>
       <c r="F24" s="8" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G24" s="10" t="n">
         <v>580</v>
@@ -2506,13 +2653,13 @@
         <v>14.04</v>
       </c>
       <c r="P24" s="10" t="n">
-        <v>4.185</v>
-      </c>
-      <c r="Q24" s="12" t="n">
-        <v>-1620</v>
-      </c>
-      <c r="R24" s="13" t="n">
-        <v>-0.1923076923076923</v>
+        <v>3.399999999999999</v>
+      </c>
+      <c r="Q24" s="39" t="n">
+        <v>264.0000000000008</v>
+      </c>
+      <c r="R24" s="40" t="n">
+        <v>0.03133903133903143</v>
       </c>
       <c r="S24" s="9" t="n">
         <v>8424</v>
@@ -2524,25 +2671,25 @@
         <v>606.785</v>
       </c>
       <c r="V24" s="10" t="n">
-        <v>601.364990234375</v>
+        <v>607.77001953125</v>
       </c>
       <c r="W24" s="38" t="n">
         <v>20.29000091552734</v>
       </c>
       <c r="X24" s="38" t="n">
-        <v>22.80999946594238</v>
+        <v>24.93000030517578</v>
       </c>
       <c r="Y24" s="14" t="n">
         <v>0.175501810962665</v>
       </c>
       <c r="Z24" s="14" t="n">
-        <v>0.240349943978385</v>
+        <v>0.2949047755251742</v>
       </c>
       <c r="AA24" s="10" t="n">
         <v>582.6986384582519</v>
       </c>
       <c r="AB24" s="10" t="n">
-        <v>586.6145758056641</v>
+        <v>588.8563188171387</v>
       </c>
       <c r="AC24" s="8" t="inlineStr">
         <is>
@@ -2690,7 +2837,7 @@
         </is>
       </c>
       <c r="F26" s="8" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G26" s="10" t="n">
         <v>658</v>
@@ -2720,13 +2867,13 @@
         <v>11.72</v>
       </c>
       <c r="P26" s="10" t="n">
-        <v>4.710000000000001</v>
+        <v>5.154999999999999</v>
       </c>
       <c r="Q26" s="12" t="n">
-        <v>-3382.000000000002</v>
+        <v>-4227.499999999999</v>
       </c>
       <c r="R26" s="13" t="n">
-        <v>-0.6075085324232086</v>
+        <v>-0.7593856655290101</v>
       </c>
       <c r="S26" s="9" t="n">
         <v>5567</v>
@@ -2738,25 +2885,25 @@
         <v>687.6799999999999</v>
       </c>
       <c r="V26" s="10" t="n">
-        <v>679.97998046875</v>
+        <v>677.1799926757812</v>
       </c>
       <c r="W26" s="38" t="n">
         <v>19.94000053405762</v>
       </c>
       <c r="X26" s="38" t="n">
-        <v>22.80999946594238</v>
+        <v>24.93000030517578</v>
       </c>
       <c r="Y26" s="14" t="n">
         <v>0.1664951108241417</v>
       </c>
       <c r="Z26" s="14" t="n">
-        <v>0.240349943978385</v>
+        <v>0.2949047755251742</v>
       </c>
       <c r="AA26" s="10" t="n">
         <v>651.1943740844727</v>
       </c>
       <c r="AB26" s="10" t="n">
-        <v>652.752537536621</v>
+        <v>655.0772604370118</v>
       </c>
       <c r="AC26" s="8" t="inlineStr">
         <is>
@@ -2789,7 +2936,7 @@
         </is>
       </c>
       <c r="F27" s="8" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G27" s="10" t="n">
         <v>245</v>
@@ -2819,13 +2966,13 @@
         <v>10.2</v>
       </c>
       <c r="P27" s="10" t="n">
-        <v>2.55</v>
-      </c>
-      <c r="Q27" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" s="40" t="n">
-        <v>0</v>
+        <v>3.66</v>
+      </c>
+      <c r="Q27" s="12" t="n">
+        <v>-111</v>
+      </c>
+      <c r="R27" s="13" t="n">
+        <v>-0.4352941176470587</v>
       </c>
       <c r="S27" s="9" t="n">
         <v>255</v>
@@ -2837,25 +2984,25 @@
         <v>257.93</v>
       </c>
       <c r="V27" s="10" t="n">
-        <v>260.0350036621094</v>
+        <v>253.3600006103516</v>
       </c>
       <c r="W27" s="38" t="n">
         <v>24.10000038146973</v>
       </c>
       <c r="X27" s="38" t="n">
-        <v>22.80999946594238</v>
+        <v>24.93000030517578</v>
       </c>
       <c r="Y27" s="14" t="n">
         <v>0.2735460547248535</v>
       </c>
       <c r="Z27" s="14" t="n">
-        <v>0.240349943978385</v>
+        <v>0.2949047755251742</v>
       </c>
       <c r="AA27" s="10" t="n">
         <v>237.4489370727539</v>
       </c>
       <c r="AB27" s="10" t="n">
-        <v>237.4594620513916</v>
+        <v>238.6874919891357</v>
       </c>
       <c r="AC27" s="8" t="inlineStr">
         <is>
@@ -2907,7 +3054,7 @@
         </is>
       </c>
       <c r="B33" s="24" t="n">
-        <v>-8092</v>
+        <v>-7874.499999999998</v>
       </c>
     </row>
     <row r="34">
@@ -2917,7 +3064,7 @@
         </is>
       </c>
       <c r="B34" s="25" t="n">
-        <v>-0.4213266687493492</v>
+        <v>-0.4100020826824949</v>
       </c>
     </row>
     <row r="35">
@@ -2953,4 +3100,846 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="41" t="inlineStr">
+        <is>
+          <t>TSLA Bear Put Debit Spread -- Position Tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="42" t="inlineStr">
+        <is>
+          <t>Last Updated: 2026-03-10 20:16:18  |  TSLA: $399.23  |  Account: IRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="43" t="inlineStr">
+        <is>
+          <t>Strategy Info</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>Structure</t>
+        </is>
+      </c>
+      <c r="B5" s="44" t="inlineStr">
+        <is>
+          <t>Bear Put Debit Spread</t>
+        </is>
+      </c>
+      <c r="C5" s="45" t="n"/>
+      <c r="D5" s="45" t="n"/>
+      <c r="E5" s="45" t="n"/>
+      <c r="F5" s="46" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>Long Leg</t>
+        </is>
+      </c>
+      <c r="B6" s="44" t="inlineStr">
+        <is>
+          <t>10x TSLA $300P @ $28.50</t>
+        </is>
+      </c>
+      <c r="C6" s="45" t="n"/>
+      <c r="D6" s="45" t="n"/>
+      <c r="E6" s="45" t="n"/>
+      <c r="F6" s="46" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>Short Leg</t>
+        </is>
+      </c>
+      <c r="B7" s="44" t="inlineStr">
+        <is>
+          <t>10x TSLA $250P @ $16.10</t>
+        </is>
+      </c>
+      <c r="C7" s="45" t="n"/>
+      <c r="D7" s="45" t="n"/>
+      <c r="E7" s="45" t="n"/>
+      <c r="F7" s="46" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>Spread Width</t>
+        </is>
+      </c>
+      <c r="B8" s="44" t="inlineStr">
+        <is>
+          <t>$50.00</t>
+        </is>
+      </c>
+      <c r="C8" s="45" t="n"/>
+      <c r="D8" s="45" t="n"/>
+      <c r="E8" s="45" t="n"/>
+      <c r="F8" s="46" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Net Debit</t>
+        </is>
+      </c>
+      <c r="B9" s="44" t="inlineStr">
+        <is>
+          <t>$12.40/share  ($12,400 total)</t>
+        </is>
+      </c>
+      <c r="C9" s="45" t="n"/>
+      <c r="D9" s="45" t="n"/>
+      <c r="E9" s="45" t="n"/>
+      <c r="F9" s="46" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>Max Profit</t>
+        </is>
+      </c>
+      <c r="B10" s="44" t="inlineStr">
+        <is>
+          <t>$37,600  (at TSLA &lt;= $250)</t>
+        </is>
+      </c>
+      <c r="C10" s="45" t="n"/>
+      <c r="D10" s="45" t="n"/>
+      <c r="E10" s="45" t="n"/>
+      <c r="F10" s="46" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>Max Loss</t>
+        </is>
+      </c>
+      <c r="B11" s="44" t="inlineStr">
+        <is>
+          <t>$12,400  (at TSLA &gt;= $300)</t>
+        </is>
+      </c>
+      <c r="C11" s="45" t="n"/>
+      <c r="D11" s="45" t="n"/>
+      <c r="E11" s="45" t="n"/>
+      <c r="F11" s="46" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>Breakeven</t>
+        </is>
+      </c>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t>$287.60</t>
+        </is>
+      </c>
+      <c r="C12" s="45" t="n"/>
+      <c r="D12" s="45" t="n"/>
+      <c r="E12" s="45" t="n"/>
+      <c r="F12" s="46" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="43" t="inlineStr">
+        <is>
+          <t>Position Detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="47" t="inlineStr">
+        <is>
+          <t>Entry Date</t>
+        </is>
+      </c>
+      <c r="B15" s="47" t="inlineStr">
+        <is>
+          <t>Expiration</t>
+        </is>
+      </c>
+      <c r="C15" s="47" t="inlineStr">
+        <is>
+          <t>DTE</t>
+        </is>
+      </c>
+      <c r="D15" s="47" t="inlineStr">
+        <is>
+          <t>Long Leg</t>
+        </is>
+      </c>
+      <c r="E15" s="47" t="inlineStr">
+        <is>
+          <t>Short Leg</t>
+        </is>
+      </c>
+      <c r="F15" s="47" t="inlineStr">
+        <is>
+          <t>Net Debit</t>
+        </is>
+      </c>
+      <c r="G15" s="47" t="inlineStr">
+        <is>
+          <t>TSLA @ Entry</t>
+        </is>
+      </c>
+      <c r="H15" s="47" t="inlineStr">
+        <is>
+          <t>TSLA Current</t>
+        </is>
+      </c>
+      <c r="I15" s="47" t="inlineStr">
+        <is>
+          <t>Spread Value</t>
+        </is>
+      </c>
+      <c r="J15" s="47" t="inlineStr">
+        <is>
+          <t>Position Value</t>
+        </is>
+      </c>
+      <c r="K15" s="47" t="inlineStr">
+        <is>
+          <t>P&amp;L ($)</t>
+        </is>
+      </c>
+      <c r="L15" s="47" t="inlineStr">
+        <is>
+          <t>P&amp;L (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>2027-01-15</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>311</v>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>$300P x10</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>$250P x10</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>392.2</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>399.2349853515625</v>
+      </c>
+      <c r="I16" s="10" t="n">
+        <v>12.20546969699686</v>
+      </c>
+      <c r="J16" s="9" t="n">
+        <v>12205.46969699686</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>-194.5303030031355</v>
+      </c>
+      <c r="L16" s="13" t="n">
+        <v>-0.01568792766154319</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="43" t="inlineStr">
+        <is>
+          <t>Net Greeks (x10 contracts x100 multiplier)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="47" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B19" s="47" t="inlineStr">
+        <is>
+          <t>Net Delta</t>
+        </is>
+      </c>
+      <c r="C19" s="47" t="inlineStr">
+        <is>
+          <t>Net Gamma</t>
+        </is>
+      </c>
+      <c r="D19" s="47" t="inlineStr">
+        <is>
+          <t>Net Theta ($/day)</t>
+        </is>
+      </c>
+      <c r="E19" s="47" t="inlineStr">
+        <is>
+          <t>Net Vega</t>
+        </is>
+      </c>
+      <c r="F19" s="47" t="inlineStr">
+        <is>
+          <t>IV (Long)</t>
+        </is>
+      </c>
+      <c r="G19" s="47" t="inlineStr">
+        <is>
+          <t>IV (Short)</t>
+        </is>
+      </c>
+      <c r="H19" s="47" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="48" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B20" s="49" t="n">
+        <v>-76.3</v>
+      </c>
+      <c r="C20" s="49" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D20" s="50" t="n">
+        <v>-16.99999999999999</v>
+      </c>
+      <c r="E20" s="51" t="n">
+        <v>29463.2</v>
+      </c>
+      <c r="F20" s="52" t="n">
+        <v>0.522</v>
+      </c>
+      <c r="G20" s="52" t="n">
+        <v>0.5526</v>
+      </c>
+      <c r="H20" s="48" t="inlineStr">
+        <is>
+          <t>ThetaData</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="B21" s="38" t="n">
+        <v>-75.50000000000001</v>
+      </c>
+      <c r="C21" s="38" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D21" s="53" t="n">
+        <v>-17.3</v>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>29601.8</v>
+      </c>
+      <c r="F21" s="54" t="n">
+        <v>0.5206</v>
+      </c>
+      <c r="G21" s="54" t="n">
+        <v>0.551</v>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>ThetaData</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="43" t="inlineStr">
+        <is>
+          <t>P&amp;L Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>Entry Cost</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>$12,400</t>
+        </is>
+      </c>
+      <c r="C24" s="45" t="n"/>
+      <c r="D24" s="46" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>Current Value</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>$12,205</t>
+        </is>
+      </c>
+      <c r="C25" s="45" t="n"/>
+      <c r="D25" s="46" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>P&amp;L ($)</t>
+        </is>
+      </c>
+      <c r="B26" s="55" t="inlineStr">
+        <is>
+          <t>$-195</t>
+        </is>
+      </c>
+      <c r="C26" s="45" t="n"/>
+      <c r="D26" s="46" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
+        <is>
+          <t>P&amp;L (%)</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>-1.6%</t>
+        </is>
+      </c>
+      <c r="C27" s="45" t="n"/>
+      <c r="D27" s="46" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>Distance to Breakeven ($287.60)</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>$+111.63  (+28.0%)</t>
+        </is>
+      </c>
+      <c r="C28" s="45" t="n"/>
+      <c r="D28" s="46" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t>Distance to Max Profit ($250)</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>$+149.23  (+37.4%)</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n"/>
+      <c r="D29" s="46" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A14:L14"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B27:D27"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="56" t="inlineStr">
+        <is>
+          <t>UPRO Long Position -- DD25%/Cool40 Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="57" t="inlineStr">
+        <is>
+          <t>Last Updated: 2026-03-10 20:16:18  |  UPRO: $110.31  |  Account: IRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="58" t="inlineStr">
+        <is>
+          <t>DD25%/Cool40 Strategy Rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>Instrument</t>
+        </is>
+      </c>
+      <c r="B5" s="44" t="inlineStr">
+        <is>
+          <t>UPRO (3x leveraged S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="C5" s="45" t="n"/>
+      <c r="D5" s="45" t="n"/>
+      <c r="E5" s="45" t="n"/>
+      <c r="F5" s="46" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>Exit Signal</t>
+        </is>
+      </c>
+      <c r="B6" s="44" t="inlineStr">
+        <is>
+          <t>UPRO closes &gt;= 25% below all-time high</t>
+        </is>
+      </c>
+      <c r="C6" s="45" t="n"/>
+      <c r="D6" s="45" t="n"/>
+      <c r="E6" s="45" t="n"/>
+      <c r="F6" s="46" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>Cooling Period</t>
+        </is>
+      </c>
+      <c r="B7" s="44" t="inlineStr">
+        <is>
+          <t>40 trading days out of market after exit</t>
+        </is>
+      </c>
+      <c r="C7" s="45" t="n"/>
+      <c r="D7" s="45" t="n"/>
+      <c r="E7" s="45" t="n"/>
+      <c r="F7" s="46" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>Re-entry</t>
+        </is>
+      </c>
+      <c r="B8" s="44" t="inlineStr">
+        <is>
+          <t>Buy UPRO after cooling period expires</t>
+        </is>
+      </c>
+      <c r="C8" s="45" t="n"/>
+      <c r="D8" s="45" t="n"/>
+      <c r="E8" s="45" t="n"/>
+      <c r="F8" s="46" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B9" s="44" t="inlineStr">
+        <is>
+          <t>COOLING state requires manual update to UPRO_POSITION dict</t>
+        </is>
+      </c>
+      <c r="C9" s="45" t="n"/>
+      <c r="D9" s="45" t="n"/>
+      <c r="E9" s="45" t="n"/>
+      <c r="F9" s="46" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="58" t="inlineStr">
+        <is>
+          <t>Position Detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="59" t="inlineStr">
+        <is>
+          <t>Shares</t>
+        </is>
+      </c>
+      <c r="B12" s="59" t="inlineStr">
+        <is>
+          <t>Entry Date</t>
+        </is>
+      </c>
+      <c r="C12" s="59" t="inlineStr">
+        <is>
+          <t>Entry Price</t>
+        </is>
+      </c>
+      <c r="D12" s="59" t="inlineStr">
+        <is>
+          <t>Cost Basis</t>
+        </is>
+      </c>
+      <c r="E12" s="59" t="inlineStr">
+        <is>
+          <t>Current Price</t>
+        </is>
+      </c>
+      <c r="F12" s="59" t="inlineStr">
+        <is>
+          <t>Current Value</t>
+        </is>
+      </c>
+      <c r="G12" s="59" t="inlineStr">
+        <is>
+          <t>P&amp;L ($)</t>
+        </is>
+      </c>
+      <c r="H12" s="59" t="inlineStr">
+        <is>
+          <t>P&amp;L (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="60" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>109.8</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>109800</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>110.3099975585938</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>110309.9975585938</v>
+      </c>
+      <c r="G13" s="39" t="n">
+        <v>509.99755859375</v>
+      </c>
+      <c r="H13" s="40" t="n">
+        <v>0.0046447865081398</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="58" t="inlineStr">
+        <is>
+          <t>DD25%/Cool40 Monitoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>All-Time High</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>$122.23</t>
+        </is>
+      </c>
+      <c r="C16" s="45" t="n"/>
+      <c r="D16" s="46" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>ATH Date</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="C17" s="45" t="n"/>
+      <c r="D17" s="46" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Current Drawdown</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>-9.8%</t>
+        </is>
+      </c>
+      <c r="C18" s="45" t="n"/>
+      <c r="D18" s="46" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>Exit Trigger Level</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>$91.67  (ATH x 0.75)</t>
+        </is>
+      </c>
+      <c r="C19" s="45" t="n"/>
+      <c r="D19" s="46" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>Distance to Exit ($)</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>$+18.64</t>
+        </is>
+      </c>
+      <c r="C20" s="45" t="n"/>
+      <c r="D20" s="46" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>Distance to Exit (%)</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>+16.9%</t>
+        </is>
+      </c>
+      <c r="C21" s="45" t="n"/>
+      <c r="D21" s="46" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B22" s="61" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="C22" s="45" t="n"/>
+      <c r="D22" s="46" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="17">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B20:D20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Sheet 5: bear spread watchlist candidates to position tracker
New bear candidates sheet with MDLZ, KHC, AIG, SBUX, CCI — includes
live pricing, spread values, bear thesis, and portfolio risk summary
alongside existing TSLA bear put spread position.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Strategies/80-Delta Call Strategy/position_tracker.xlsx
+++ b/Strategies/80-Delta Call Strategy/position_tracker.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCS Paper Trades" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TSLA Bear Put Spread" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UPRO DD25-Cool40" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear Spread Candidates" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
     <numFmt numFmtId="167" formatCode="$#,##0.00"/>
     <numFmt numFmtId="168" formatCode="0.1%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -121,8 +122,14 @@
       <color rgb="00006100"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="009C6500"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -201,6 +208,12 @@
         <bgColor rgb="002E7D32"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -248,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -413,6 +426,10 @@
     <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -820,14 +837,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last Updated: 2026-03-10 20:16:17  |  SPY: $677.18  |  QQQ: $607.77</t>
+          <t>Last Updated: 2026-03-11 15:40:55  |  SPY: $676.09  |  QQQ: $607.65</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>SPY SMA200: $655.08 (+3.4%)  |  QQQ SMA200: $588.86 (+3.2%)</t>
+          <t>SPY SMA200: $655.57 (+3.1%)  |  QQQ SMA200: $589.33 (+3.1%)</t>
         </is>
       </c>
     </row>
@@ -1169,31 +1186,31 @@
         <v>640</v>
       </c>
       <c r="P21" s="10" t="n">
-        <v>39.6072213876563</v>
+        <v>38.70923761694712</v>
       </c>
       <c r="Q21" s="9" t="n">
-        <v>39607.2213876563</v>
+        <v>38709.23761694712</v>
       </c>
       <c r="R21" s="11" t="n">
-        <v>0.6739013349292748</v>
+        <v>0.6678594445532715</v>
       </c>
       <c r="S21" s="7" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="T21" s="12" t="n">
-        <v>-11992.7786123437</v>
+        <v>-12890.76238305288</v>
       </c>
       <c r="U21" s="13" t="n">
-        <v>-0.2324181901616997</v>
+        <v>-0.2498209764157535</v>
       </c>
       <c r="V21" s="10" t="n">
         <v>77.40000000000001</v>
       </c>
       <c r="W21" s="14" t="n">
-        <v>0.9541890919952779</v>
+        <v>0.9995227177017264</v>
       </c>
       <c r="X21" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Y21" s="8" t="inlineStr">
         <is>
@@ -1201,7 +1218,7 @@
         </is>
       </c>
       <c r="Z21" s="7" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AA21" s="8" t="inlineStr">
         <is>
@@ -1264,31 +1281,31 @@
         <v>640</v>
       </c>
       <c r="P22" s="18" t="n">
-        <v>42.89079616610218</v>
+        <v>41.91379480841061</v>
       </c>
       <c r="Q22" s="17" t="n">
-        <v>42890.79616610217</v>
+        <v>41913.79480841061</v>
       </c>
       <c r="R22" s="19" t="n">
-        <v>0.7406307270636951</v>
+        <v>0.7350386317824302</v>
       </c>
       <c r="S22" s="15" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="T22" s="12" t="n">
-        <v>-12519.20383389783</v>
+        <v>-13496.20519158939</v>
       </c>
       <c r="U22" s="13" t="n">
-        <v>-0.2259376255892045</v>
+        <v>-0.2435698464462982</v>
       </c>
       <c r="V22" s="18" t="n">
         <v>83.11499999999999</v>
       </c>
       <c r="W22" s="20" t="n">
-        <v>0.9378283321699716</v>
+        <v>0.98299868527585</v>
       </c>
       <c r="X22" s="15" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Y22" s="16" t="inlineStr">
         <is>
@@ -1296,7 +1313,7 @@
         </is>
       </c>
       <c r="Z22" s="15" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AA22" s="16" t="inlineStr">
         <is>
@@ -1359,31 +1376,31 @@
         <v>640</v>
       </c>
       <c r="P23" s="10" t="n">
-        <v>36.8934173771782</v>
+        <v>35.92453442496299</v>
       </c>
       <c r="Q23" s="9" t="n">
-        <v>36893.41737717819</v>
+        <v>35924.53442496299</v>
       </c>
       <c r="R23" s="11" t="n">
-        <v>0.7189281090771118</v>
+        <v>0.7124948451141824</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="T23" s="12" t="n">
-        <v>-12806.58262282181</v>
+        <v>-13775.46557503701</v>
       </c>
       <c r="U23" s="13" t="n">
-        <v>-0.2576777187690504</v>
+        <v>-0.2771723455741855</v>
       </c>
       <c r="V23" s="10" t="n">
         <v>74.55000000000001</v>
       </c>
       <c r="W23" s="14" t="n">
-        <v>1.020685675112214</v>
+        <v>1.075183469829389</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Y23" s="8" t="inlineStr">
         <is>
@@ -1391,7 +1408,7 @@
         </is>
       </c>
       <c r="Z23" s="7" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="AA23" s="8" t="inlineStr">
         <is>
@@ -1454,31 +1471,31 @@
         <v>641</v>
       </c>
       <c r="P24" s="18" t="n">
-        <v>42.83815801513327</v>
+        <v>41.91129644458545</v>
       </c>
       <c r="Q24" s="17" t="n">
-        <v>42838.15801513327</v>
+        <v>41911.29644458544</v>
       </c>
       <c r="R24" s="19" t="n">
-        <v>0.7024381907695142</v>
+        <v>0.6967692513541669</v>
       </c>
       <c r="S24" s="15" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="T24" s="12" t="n">
-        <v>-8921.841984866725</v>
+        <v>-9848.703555414555</v>
       </c>
       <c r="U24" s="13" t="n">
-        <v>-0.1723694355654313</v>
+        <v>-0.190276343806309</v>
       </c>
       <c r="V24" s="18" t="n">
         <v>77.64</v>
       </c>
       <c r="W24" s="20" t="n">
-        <v>0.8124028575778728</v>
+        <v>0.8524838548636778</v>
       </c>
       <c r="X24" s="15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Y24" s="16" t="inlineStr">
         <is>
@@ -1486,7 +1503,7 @@
         </is>
       </c>
       <c r="Z24" s="15" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="AA24" s="16" t="inlineStr">
         <is>
@@ -1549,31 +1566,31 @@
         <v>653</v>
       </c>
       <c r="P25" s="10" t="n">
-        <v>65.0868710932462</v>
+        <v>64.02577842951996</v>
       </c>
       <c r="Q25" s="9" t="n">
-        <v>32543.4355466231</v>
+        <v>32012.88921475998</v>
       </c>
       <c r="R25" s="11" t="n">
-        <v>0.8482701381105086</v>
+        <v>0.8450077005638217</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="T25" s="12" t="n">
-        <v>-3296.564453376908</v>
+        <v>-3827.110785240027</v>
       </c>
       <c r="U25" s="13" t="n">
-        <v>-0.09198003497145368</v>
+        <v>-0.1067832250345988</v>
       </c>
       <c r="V25" s="10" t="n">
         <v>107.52</v>
       </c>
       <c r="W25" s="14" t="n">
-        <v>0.6519460560020209</v>
+        <v>0.6793235886754396</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y25" s="8" t="inlineStr">
         <is>
@@ -1581,7 +1598,7 @@
         </is>
       </c>
       <c r="Z25" s="7" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AA25" s="8" t="inlineStr">
         <is>
@@ -1644,31 +1661,31 @@
         <v>587</v>
       </c>
       <c r="P26" s="18" t="n">
-        <v>67.60096608682267</v>
+        <v>67.38222000467931</v>
       </c>
       <c r="Q26" s="17" t="n">
-        <v>33800.48304341133</v>
+        <v>33691.11000233966</v>
       </c>
       <c r="R26" s="19" t="n">
-        <v>0.8921530107565758</v>
+        <v>0.8925865828352806</v>
       </c>
       <c r="S26" s="15" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="T26" s="12" t="n">
-        <v>-1934.516956588668</v>
+        <v>-2043.889997660342</v>
       </c>
       <c r="U26" s="13" t="n">
-        <v>-0.05413507644014737</v>
+        <v>-0.05719574640157676</v>
       </c>
       <c r="V26" s="18" t="n">
         <v>107.205</v>
       </c>
       <c r="W26" s="20" t="n">
-        <v>0.5858501173239486</v>
+        <v>0.590998337433157</v>
       </c>
       <c r="X26" s="15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y26" s="16" t="inlineStr">
         <is>
@@ -1676,7 +1693,7 @@
         </is>
       </c>
       <c r="Z26" s="15" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AA26" s="16" t="inlineStr">
         <is>
@@ -1728,7 +1745,7 @@
         </is>
       </c>
       <c r="B32" s="23" t="n">
-        <v>228573.5115361044</v>
+        <v>224162.8625120058</v>
       </c>
     </row>
     <row r="33">
@@ -1738,7 +1755,7 @@
         </is>
       </c>
       <c r="B33" s="24" t="n">
-        <v>-51471.48846389563</v>
+        <v>-55882.13748799422</v>
       </c>
     </row>
     <row r="34">
@@ -1748,7 +1765,7 @@
         </is>
       </c>
       <c r="B34" s="25" t="n">
-        <v>-0.1837972056772863</v>
+        <v>-0.1995469924047715</v>
       </c>
     </row>
     <row r="35">
@@ -1758,7 +1775,7 @@
         </is>
       </c>
       <c r="B35" s="26" t="n">
-        <v>3706.109936273138</v>
+        <v>3680.959314503602</v>
       </c>
     </row>
     <row r="36">
@@ -1768,7 +1785,7 @@
         </is>
       </c>
       <c r="B36" s="26" t="n">
-        <v>3706</v>
+        <v>3680</v>
       </c>
     </row>
     <row r="38">
@@ -1827,7 +1844,7 @@
         </is>
       </c>
       <c r="B40" s="9" t="n">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
@@ -1835,19 +1852,19 @@
         </is>
       </c>
       <c r="D40" s="8" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E40" s="11" t="n">
-        <v>0.8001781124678849</v>
+        <v>0.8008157555494608</v>
       </c>
       <c r="F40" s="10" t="n">
-        <v>84.899162985239</v>
+        <v>84.59498860519562</v>
       </c>
       <c r="G40" s="9" t="n">
-        <v>84899.162985239</v>
+        <v>84594.98860519563</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>42449.5814926195</v>
+        <v>42297.49430259781</v>
       </c>
     </row>
     <row r="41">
@@ -1865,19 +1882,19 @@
         </is>
       </c>
       <c r="D41" s="8" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E41" s="11" t="n">
-        <v>0.8004037738276757</v>
+        <v>0.8006321034977426</v>
       </c>
       <c r="F41" s="10" t="n">
-        <v>76.24616385754177</v>
+        <v>75.99168139180551</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>76246.16385754177</v>
+        <v>75991.68139180551</v>
       </c>
       <c r="H41" s="9" t="n">
-        <v>38123.08192877089</v>
+        <v>37995.84069590276</v>
       </c>
     </row>
   </sheetData>
@@ -1956,7 +1973,7 @@
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
         <is>
-          <t>Last Updated: 2026-03-10 20:16:17  |  SPY: $677.18  |  QQQ: $607.77  |  PAPER TRADING - NOT REAL MONEY</t>
+          <t>Last Updated: 2026-03-11 15:40:56  |  SPY: $676.09  |  QQQ: $607.65  |  PAPER TRADING - NOT REAL MONEY</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2541,7 @@
         </is>
       </c>
       <c r="F23" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G23" s="10" t="n">
         <v>657</v>
@@ -2554,13 +2571,13 @@
         <v>9.92</v>
       </c>
       <c r="P23" s="10" t="n">
-        <v>4.38</v>
+        <v>3.31</v>
       </c>
       <c r="Q23" s="12" t="n">
-        <v>-3800</v>
+        <v>-1659.999999999999</v>
       </c>
       <c r="R23" s="13" t="n">
-        <v>-0.7661290322580645</v>
+        <v>-0.3346774193548385</v>
       </c>
       <c r="S23" s="9" t="n">
         <v>4960</v>
@@ -2572,25 +2589,25 @@
         <v>686.8</v>
       </c>
       <c r="V23" s="10" t="n">
-        <v>677.1799926757812</v>
+        <v>676.0900268554688</v>
       </c>
       <c r="W23" s="38" t="n">
         <v>19.92000007629395</v>
       </c>
       <c r="X23" s="38" t="n">
-        <v>24.93000030517578</v>
+        <v>24.92000007629395</v>
       </c>
       <c r="Y23" s="14" t="n">
         <v>0.1659804310259251</v>
       </c>
       <c r="Z23" s="14" t="n">
-        <v>0.2949047755251742</v>
+        <v>0.2946474356260659</v>
       </c>
       <c r="AA23" s="10" t="n">
         <v>648.5776251220703</v>
       </c>
       <c r="AB23" s="10" t="n">
-        <v>655.0772604370118</v>
+        <v>655.5674285888672</v>
       </c>
       <c r="AC23" s="8" t="inlineStr">
         <is>
@@ -2623,7 +2640,7 @@
         </is>
       </c>
       <c r="F24" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G24" s="10" t="n">
         <v>580</v>
@@ -2653,13 +2670,13 @@
         <v>14.04</v>
       </c>
       <c r="P24" s="10" t="n">
-        <v>3.399999999999999</v>
+        <v>2.11</v>
       </c>
       <c r="Q24" s="39" t="n">
-        <v>264.0000000000008</v>
+        <v>3360</v>
       </c>
       <c r="R24" s="40" t="n">
-        <v>0.03133903133903143</v>
+        <v>0.3988603988603989</v>
       </c>
       <c r="S24" s="9" t="n">
         <v>8424</v>
@@ -2671,25 +2688,25 @@
         <v>606.785</v>
       </c>
       <c r="V24" s="10" t="n">
-        <v>607.77001953125</v>
+        <v>607.6500244140625</v>
       </c>
       <c r="W24" s="38" t="n">
         <v>20.29000091552734</v>
       </c>
       <c r="X24" s="38" t="n">
-        <v>24.93000030517578</v>
+        <v>24.92000007629395</v>
       </c>
       <c r="Y24" s="14" t="n">
         <v>0.175501810962665</v>
       </c>
       <c r="Z24" s="14" t="n">
-        <v>0.2949047755251742</v>
+        <v>0.2946474356260659</v>
       </c>
       <c r="AA24" s="10" t="n">
         <v>582.6986384582519</v>
       </c>
       <c r="AB24" s="10" t="n">
-        <v>588.8563188171387</v>
+        <v>589.3337240600586</v>
       </c>
       <c r="AC24" s="8" t="inlineStr">
         <is>
@@ -2837,7 +2854,7 @@
         </is>
       </c>
       <c r="F26" s="8" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G26" s="10" t="n">
         <v>658</v>
@@ -2867,13 +2884,13 @@
         <v>11.72</v>
       </c>
       <c r="P26" s="10" t="n">
-        <v>5.154999999999999</v>
+        <v>4.565</v>
       </c>
       <c r="Q26" s="12" t="n">
-        <v>-4227.499999999999</v>
+        <v>-3106.5</v>
       </c>
       <c r="R26" s="13" t="n">
-        <v>-0.7593856655290101</v>
+        <v>-0.5580204778156995</v>
       </c>
       <c r="S26" s="9" t="n">
         <v>5567</v>
@@ -2885,25 +2902,25 @@
         <v>687.6799999999999</v>
       </c>
       <c r="V26" s="10" t="n">
-        <v>677.1799926757812</v>
+        <v>676.0900268554688</v>
       </c>
       <c r="W26" s="38" t="n">
         <v>19.94000053405762</v>
       </c>
       <c r="X26" s="38" t="n">
-        <v>24.93000030517578</v>
+        <v>24.92000007629395</v>
       </c>
       <c r="Y26" s="14" t="n">
         <v>0.1664951108241417</v>
       </c>
       <c r="Z26" s="14" t="n">
-        <v>0.2949047755251742</v>
+        <v>0.2946474356260659</v>
       </c>
       <c r="AA26" s="10" t="n">
         <v>651.1943740844727</v>
       </c>
       <c r="AB26" s="10" t="n">
-        <v>655.0772604370118</v>
+        <v>655.5674285888672</v>
       </c>
       <c r="AC26" s="8" t="inlineStr">
         <is>
@@ -2936,7 +2953,7 @@
         </is>
       </c>
       <c r="F27" s="8" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G27" s="10" t="n">
         <v>245</v>
@@ -2966,13 +2983,13 @@
         <v>10.2</v>
       </c>
       <c r="P27" s="10" t="n">
-        <v>3.66</v>
+        <v>3.415000000000001</v>
       </c>
       <c r="Q27" s="12" t="n">
-        <v>-111</v>
+        <v>-86.50000000000007</v>
       </c>
       <c r="R27" s="13" t="n">
-        <v>-0.4352941176470587</v>
+        <v>-0.33921568627451</v>
       </c>
       <c r="S27" s="9" t="n">
         <v>255</v>
@@ -2984,25 +3001,25 @@
         <v>257.93</v>
       </c>
       <c r="V27" s="10" t="n">
-        <v>253.3600006103516</v>
+        <v>252.5200042724609</v>
       </c>
       <c r="W27" s="38" t="n">
         <v>24.10000038146973</v>
       </c>
       <c r="X27" s="38" t="n">
-        <v>24.93000030517578</v>
+        <v>24.92000007629395</v>
       </c>
       <c r="Y27" s="14" t="n">
         <v>0.2735460547248535</v>
       </c>
       <c r="Z27" s="14" t="n">
-        <v>0.2949047755251742</v>
+        <v>0.2946474356260659</v>
       </c>
       <c r="AA27" s="10" t="n">
         <v>237.4489370727539</v>
       </c>
       <c r="AB27" s="10" t="n">
-        <v>238.6874919891357</v>
+        <v>238.9431359863281</v>
       </c>
       <c r="AC27" s="8" t="inlineStr">
         <is>
@@ -3054,7 +3071,7 @@
         </is>
       </c>
       <c r="B33" s="24" t="n">
-        <v>-7874.499999999998</v>
+        <v>-1492.999999999999</v>
       </c>
     </row>
     <row r="34">
@@ -3064,7 +3081,7 @@
         </is>
       </c>
       <c r="B34" s="25" t="n">
-        <v>-0.4100020826824949</v>
+        <v>-0.07773612412787663</v>
       </c>
     </row>
     <row r="35">
@@ -3135,7 +3152,7 @@
     <row r="2">
       <c r="A2" s="42" t="inlineStr">
         <is>
-          <t>Last Updated: 2026-03-10 20:16:18  |  TSLA: $399.23  |  Account: IRA</t>
+          <t>Last Updated: 2026-03-11 15:40:56  |  TSLA: $407.98  |  Account: IRA</t>
         </is>
       </c>
     </row>
@@ -3355,7 +3372,7 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
@@ -3374,19 +3391,19 @@
         <v>392.2</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>399.2349853515625</v>
+        <v>407.9779968261719</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>12.20546969699686</v>
+        <v>0.9758656744633745</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>12205.46969699686</v>
+        <v>975.8656744633745</v>
       </c>
       <c r="K16" s="12" t="n">
-        <v>-194.5303030031355</v>
+        <v>-11424.13432553663</v>
       </c>
       <c r="L16" s="13" t="n">
-        <v>-0.01568792766154319</v>
+        <v>-0.9213011552852118</v>
       </c>
     </row>
     <row r="18">
@@ -3471,30 +3488,30 @@
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B21" s="38" t="n">
-        <v>-75.50000000000001</v>
+        <v>-28.59279934394488</v>
       </c>
       <c r="C21" s="38" t="n">
-        <v>0.4</v>
+        <v>0.7793169074627853</v>
       </c>
       <c r="D21" s="53" t="n">
-        <v>-17.3</v>
+        <v>-6.458575827832616</v>
       </c>
       <c r="E21" s="11" t="n">
-        <v>29601.8</v>
+        <v>234.0086000778251</v>
       </c>
       <c r="F21" s="54" t="n">
-        <v>0.5206</v>
+        <v>0.2124102197265625</v>
       </c>
       <c r="G21" s="54" t="n">
-        <v>0.551</v>
+        <v>0.2124102197265625</v>
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>ThetaData</t>
+          <t>BS estimate</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3544,7 @@
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>$12,205</t>
+          <t>$976</t>
         </is>
       </c>
       <c r="C25" s="45" t="n"/>
@@ -3541,7 +3558,7 @@
       </c>
       <c r="B26" s="55" t="inlineStr">
         <is>
-          <t>$-195</t>
+          <t>$-11,424</t>
         </is>
       </c>
       <c r="C26" s="45" t="n"/>
@@ -3555,7 +3572,7 @@
       </c>
       <c r="B27" s="22" t="inlineStr">
         <is>
-          <t>-1.6%</t>
+          <t>-92.1%</t>
         </is>
       </c>
       <c r="C27" s="45" t="n"/>
@@ -3569,7 +3586,7 @@
       </c>
       <c r="B28" s="22" t="inlineStr">
         <is>
-          <t>$+111.63  (+28.0%)</t>
+          <t>$+120.38  (+29.5%)</t>
         </is>
       </c>
       <c r="C28" s="45" t="n"/>
@@ -3583,7 +3600,7 @@
       </c>
       <c r="B29" s="22" t="inlineStr">
         <is>
-          <t>$+149.23  (+37.4%)</t>
+          <t>$+157.98  (+38.7%)</t>
         </is>
       </c>
       <c r="C29" s="45" t="n"/>
@@ -3647,7 +3664,7 @@
     <row r="2">
       <c r="A2" s="57" t="inlineStr">
         <is>
-          <t>Last Updated: 2026-03-10 20:16:18  |  UPRO: $110.31  |  Account: IRA</t>
+          <t>Last Updated: 2026-03-11 15:40:57  |  UPRO: $109.81  |  Account: IRA</t>
         </is>
       </c>
     </row>
@@ -3803,16 +3820,16 @@
         <v>109800</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>110.3099975585938</v>
+        <v>109.8099975585938</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>110309.9975585938</v>
+        <v>109809.9975585938</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>509.99755859375</v>
+        <v>9.99755859375</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>0.0046447865081398</v>
+        <v>9.10524462090164e-05</v>
       </c>
     </row>
     <row r="15">
@@ -3858,7 +3875,7 @@
       </c>
       <c r="B18" s="22" t="inlineStr">
         <is>
-          <t>-9.8%</t>
+          <t>-10.2%</t>
         </is>
       </c>
       <c r="C18" s="45" t="n"/>
@@ -3886,7 +3903,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>$+18.64</t>
+          <t>$+18.14</t>
         </is>
       </c>
       <c r="C20" s="45" t="n"/>
@@ -3900,7 +3917,7 @@
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>+16.9%</t>
+          <t>+16.5%</t>
         </is>
       </c>
       <c r="C21" s="45" t="n"/>
@@ -3942,4 +3959,608 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="41" t="inlineStr">
+        <is>
+          <t>Bear Put Spread Candidates -- Watchlist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="42" t="inlineStr">
+        <is>
+          <t>Last Updated: 2026-03-11 15:40:59  |  Screened: 2026-03-11  |  Source: IC-derived scoring + GuruFocus</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="43" t="inlineStr">
+        <is>
+          <t>Candidate Overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="47" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C5" s="47" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="D5" s="47" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E5" s="47" t="inlineStr">
+        <is>
+          <t>Long Put</t>
+        </is>
+      </c>
+      <c r="F5" s="47" t="inlineStr">
+        <is>
+          <t>Short Put</t>
+        </is>
+      </c>
+      <c r="G5" s="47" t="inlineStr">
+        <is>
+          <t>Exp</t>
+        </is>
+      </c>
+      <c r="H5" s="47" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="I5" s="47" t="inlineStr">
+        <is>
+          <t>R:R</t>
+        </is>
+      </c>
+      <c r="J5" s="47" t="inlineStr">
+        <is>
+          <t>Current Price</t>
+        </is>
+      </c>
+      <c r="K5" s="47" t="inlineStr">
+        <is>
+          <t>Spread Value</t>
+        </is>
+      </c>
+      <c r="L5" s="47" t="inlineStr">
+        <is>
+          <t>Est. Debit</t>
+        </is>
+      </c>
+      <c r="M5" s="47" t="inlineStr">
+        <is>
+          <t>Max Loss/Ct</t>
+        </is>
+      </c>
+      <c r="N5" s="47" t="inlineStr">
+        <is>
+          <t>Max Profit/Ct</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>MDLZ</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Mondelez International</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="D6" s="62" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>$55P</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>$27.5P</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>2027-01-15</t>
+        </is>
+      </c>
+      <c r="H6" s="38" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="J6" s="53" t="n">
+        <v>55.46500015258789</v>
+      </c>
+      <c r="K6" s="10" t="n">
+        <v>5.299925828150436</v>
+      </c>
+      <c r="L6" s="10" t="n">
+        <v>5.299925828150436</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>529.9925828150436</v>
+      </c>
+      <c r="N6" s="9" t="n">
+        <v>2220.007417184956</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>KHC</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Kraft Heinz</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="D7" s="62" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>$22.5P</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>$12.5P</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>2027-01-15</t>
+        </is>
+      </c>
+      <c r="H7" s="38" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="J7" s="53" t="n">
+        <v>23.20999908447266</v>
+      </c>
+      <c r="K7" s="10" t="n">
+        <v>2.202785509422638</v>
+      </c>
+      <c r="L7" s="10" t="n">
+        <v>2.202785509422638</v>
+      </c>
+      <c r="M7" s="9" t="n">
+        <v>220.2785509422638</v>
+      </c>
+      <c r="N7" s="9" t="n">
+        <v>779.7214490577362</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>AIG</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>American International Group</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D8" s="62" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>$77.5P</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>$37.5P</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>2027-01-15</t>
+        </is>
+      </c>
+      <c r="H8" s="38" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="J8" s="53" t="n">
+        <v>77.83000183105469</v>
+      </c>
+      <c r="K8" s="10" t="n">
+        <v>11.48804953094305</v>
+      </c>
+      <c r="L8" s="10" t="n">
+        <v>11.48804953094305</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>1148.804953094305</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>2851.195046905695</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Starbucks</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D9" s="62" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>$100P</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>$50P</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>2027-01-15</t>
+        </is>
+      </c>
+      <c r="H9" s="38" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="J9" s="53" t="n">
+        <v>101.2050018310547</v>
+      </c>
+      <c r="K9" s="10" t="n">
+        <v>11.60000803443361</v>
+      </c>
+      <c r="L9" s="10" t="n">
+        <v>11.60000803443361</v>
+      </c>
+      <c r="M9" s="9" t="n">
+        <v>1160.000803443361</v>
+      </c>
+      <c r="N9" s="9" t="n">
+        <v>3839.999196556639</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>CCI</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Crown Castle</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="D10" s="62" t="inlineStr">
+        <is>
+          <t>WATCHLIST</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>$87.5P</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>$45P</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>2027-01-15</t>
+        </is>
+      </c>
+      <c r="H10" s="38" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="J10" s="53" t="n">
+        <v>87.59999847412109</v>
+      </c>
+      <c r="K10" s="10" t="n">
+        <v>10.40465458484316</v>
+      </c>
+      <c r="L10" s="10" t="n">
+        <v>10.40465458484316</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>1040.465458484316</v>
+      </c>
+      <c r="N10" s="9" t="n">
+        <v>3209.534541515684</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="43" t="inlineStr">
+        <is>
+          <t>Bear Thesis Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>MDLZ</t>
+        </is>
+      </c>
+      <c r="B13" s="63" t="inlineStr">
+        <is>
+          <t>Cocoa hedge trap, volume decline 4.8%, FY26 guidance below Street</t>
+        </is>
+      </c>
+      <c r="C13" s="45" t="n"/>
+      <c r="D13" s="45" t="n"/>
+      <c r="E13" s="45" t="n"/>
+      <c r="F13" s="45" t="n"/>
+      <c r="G13" s="45" t="n"/>
+      <c r="H13" s="45" t="n"/>
+      <c r="I13" s="45" t="n"/>
+      <c r="J13" s="45" t="n"/>
+      <c r="K13" s="45" t="n"/>
+      <c r="L13" s="45" t="n"/>
+      <c r="M13" s="45" t="n"/>
+      <c r="N13" s="46" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>KHC</t>
+        </is>
+      </c>
+      <c r="B14" s="63" t="inlineStr">
+        <is>
+          <t>Revenue declining, split paused, FY26 EPS $2.03 vs Street $2.68</t>
+        </is>
+      </c>
+      <c r="C14" s="45" t="n"/>
+      <c r="D14" s="45" t="n"/>
+      <c r="E14" s="45" t="n"/>
+      <c r="F14" s="45" t="n"/>
+      <c r="G14" s="45" t="n"/>
+      <c r="H14" s="45" t="n"/>
+      <c r="I14" s="45" t="n"/>
+      <c r="J14" s="45" t="n"/>
+      <c r="K14" s="45" t="n"/>
+      <c r="L14" s="45" t="n"/>
+      <c r="M14" s="45" t="n"/>
+      <c r="N14" s="46" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>AIG</t>
+        </is>
+      </c>
+      <c r="B15" s="63" t="inlineStr">
+        <is>
+          <t>CEO transition, underwriting headwinds, cat exposure</t>
+        </is>
+      </c>
+      <c r="C15" s="45" t="n"/>
+      <c r="D15" s="45" t="n"/>
+      <c r="E15" s="45" t="n"/>
+      <c r="F15" s="45" t="n"/>
+      <c r="G15" s="45" t="n"/>
+      <c r="H15" s="45" t="n"/>
+      <c r="I15" s="45" t="n"/>
+      <c r="J15" s="45" t="n"/>
+      <c r="K15" s="45" t="n"/>
+      <c r="L15" s="45" t="n"/>
+      <c r="M15" s="45" t="n"/>
+      <c r="N15" s="46" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="B16" s="63" t="inlineStr">
+        <is>
+          <t>Consumer weakness, high FwdPE 44x, turnaround uncertainty</t>
+        </is>
+      </c>
+      <c r="C16" s="45" t="n"/>
+      <c r="D16" s="45" t="n"/>
+      <c r="E16" s="45" t="n"/>
+      <c r="F16" s="45" t="n"/>
+      <c r="G16" s="45" t="n"/>
+      <c r="H16" s="45" t="n"/>
+      <c r="I16" s="45" t="n"/>
+      <c r="J16" s="45" t="n"/>
+      <c r="K16" s="45" t="n"/>
+      <c r="L16" s="45" t="n"/>
+      <c r="M16" s="45" t="n"/>
+      <c r="N16" s="46" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>CCI</t>
+        </is>
+      </c>
+      <c r="B17" s="63" t="inlineStr">
+        <is>
+          <t>REIT rate-sensitive, GFV=9, tower growth slowing</t>
+        </is>
+      </c>
+      <c r="C17" s="45" t="n"/>
+      <c r="D17" s="45" t="n"/>
+      <c r="E17" s="45" t="n"/>
+      <c r="F17" s="45" t="n"/>
+      <c r="G17" s="45" t="n"/>
+      <c r="H17" s="45" t="n"/>
+      <c r="I17" s="45" t="n"/>
+      <c r="J17" s="45" t="n"/>
+      <c r="K17" s="45" t="n"/>
+      <c r="L17" s="45" t="n"/>
+      <c r="M17" s="45" t="n"/>
+      <c r="N17" s="46" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="43" t="inlineStr">
+        <is>
+          <t>Portfolio Risk Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>TSLA Bear Put Spread (existing)</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>$12,400</t>
+        </is>
+      </c>
+      <c r="C20" s="45" t="n"/>
+      <c r="D20" s="46" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>Candidates (est. 1 contract each)</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>$4,100</t>
+        </is>
+      </c>
+      <c r="C21" s="45" t="n"/>
+      <c r="D21" s="46" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Total Bear Overlay Risk</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>$16,500</t>
+        </is>
+      </c>
+      <c r="C22" s="45" t="n"/>
+      <c r="D22" s="46" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="B14:N14"/>
+    <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A4:N4"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="B17:N17"/>
+    <mergeCell ref="B13:N13"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B15:N15"/>
+    <mergeCell ref="B16:N16"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>